<commit_message>
Relabel workbooks: inline dropdowns, unlocked sheets, checkbox-ready Unsure column
</commit_message>
<xml_diff>
--- a/reannotation_2026-09-27/outputs/relabel/annotator_1_Laiba.xlsx
+++ b/reannotation_2026-09-27/outputs/relabel/annotator_1_Laiba.xlsx
@@ -8,7 +8,6 @@
   </bookViews>
   <sheets>
     <sheet name="Laiba" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="_lists" sheetId="2" state="hidden" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -537,7 +536,9 @@
       </c>
       <c r="D2" s="4" t="inlineStr"/>
       <c r="E2" s="4" t="inlineStr"/>
-      <c r="F2" s="4" t="inlineStr"/>
+      <c r="F2" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="G2" s="4" t="inlineStr"/>
     </row>
     <row r="3">
@@ -556,7 +557,9 @@
       </c>
       <c r="D3" s="4" t="inlineStr"/>
       <c r="E3" s="4" t="inlineStr"/>
-      <c r="F3" s="4" t="inlineStr"/>
+      <c r="F3" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="G3" s="4" t="inlineStr"/>
     </row>
     <row r="4">
@@ -575,7 +578,9 @@
       </c>
       <c r="D4" s="4" t="inlineStr"/>
       <c r="E4" s="4" t="inlineStr"/>
-      <c r="F4" s="4" t="inlineStr"/>
+      <c r="F4" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="G4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
@@ -594,7 +599,9 @@
       </c>
       <c r="D5" s="4" t="inlineStr"/>
       <c r="E5" s="4" t="inlineStr"/>
-      <c r="F5" s="4" t="inlineStr"/>
+      <c r="F5" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="G5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
@@ -613,7 +620,9 @@
       </c>
       <c r="D6" s="4" t="inlineStr"/>
       <c r="E6" s="4" t="inlineStr"/>
-      <c r="F6" s="4" t="inlineStr"/>
+      <c r="F6" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="G6" s="4" t="inlineStr"/>
     </row>
     <row r="7">
@@ -632,7 +641,9 @@
       </c>
       <c r="D7" s="4" t="inlineStr"/>
       <c r="E7" s="4" t="inlineStr"/>
-      <c r="F7" s="4" t="inlineStr"/>
+      <c r="F7" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="G7" s="4" t="inlineStr"/>
     </row>
     <row r="8">
@@ -651,7 +662,9 @@
       </c>
       <c r="D8" s="4" t="inlineStr"/>
       <c r="E8" s="4" t="inlineStr"/>
-      <c r="F8" s="4" t="inlineStr"/>
+      <c r="F8" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="G8" s="4" t="inlineStr"/>
     </row>
     <row r="9">
@@ -670,7 +683,9 @@
       </c>
       <c r="D9" s="4" t="inlineStr"/>
       <c r="E9" s="4" t="inlineStr"/>
-      <c r="F9" s="4" t="inlineStr"/>
+      <c r="F9" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="G9" s="4" t="inlineStr"/>
     </row>
     <row r="10">
@@ -689,7 +704,9 @@
       </c>
       <c r="D10" s="4" t="inlineStr"/>
       <c r="E10" s="4" t="inlineStr"/>
-      <c r="F10" s="4" t="inlineStr"/>
+      <c r="F10" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="G10" s="4" t="inlineStr"/>
     </row>
     <row r="11">
@@ -708,7 +725,9 @@
       </c>
       <c r="D11" s="4" t="inlineStr"/>
       <c r="E11" s="4" t="inlineStr"/>
-      <c r="F11" s="4" t="inlineStr"/>
+      <c r="F11" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="G11" s="4" t="inlineStr"/>
     </row>
     <row r="12">
@@ -727,7 +746,9 @@
       </c>
       <c r="D12" s="4" t="inlineStr"/>
       <c r="E12" s="4" t="inlineStr"/>
-      <c r="F12" s="4" t="inlineStr"/>
+      <c r="F12" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="G12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
@@ -746,7 +767,9 @@
       </c>
       <c r="D13" s="4" t="inlineStr"/>
       <c r="E13" s="4" t="inlineStr"/>
-      <c r="F13" s="4" t="inlineStr"/>
+      <c r="F13" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="G13" s="4" t="inlineStr"/>
     </row>
     <row r="14">
@@ -765,7 +788,9 @@
       </c>
       <c r="D14" s="4" t="inlineStr"/>
       <c r="E14" s="4" t="inlineStr"/>
-      <c r="F14" s="4" t="inlineStr"/>
+      <c r="F14" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="G14" s="4" t="inlineStr"/>
     </row>
     <row r="15">
@@ -784,7 +809,9 @@
       </c>
       <c r="D15" s="4" t="inlineStr"/>
       <c r="E15" s="4" t="inlineStr"/>
-      <c r="F15" s="4" t="inlineStr"/>
+      <c r="F15" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="G15" s="4" t="inlineStr"/>
     </row>
     <row r="16">
@@ -803,7 +830,9 @@
       </c>
       <c r="D16" s="4" t="inlineStr"/>
       <c r="E16" s="4" t="inlineStr"/>
-      <c r="F16" s="4" t="inlineStr"/>
+      <c r="F16" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="G16" s="4" t="inlineStr"/>
     </row>
     <row r="17">
@@ -822,7 +851,9 @@
       </c>
       <c r="D17" s="4" t="inlineStr"/>
       <c r="E17" s="4" t="inlineStr"/>
-      <c r="F17" s="4" t="inlineStr"/>
+      <c r="F17" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="G17" s="4" t="inlineStr"/>
     </row>
     <row r="18">
@@ -841,7 +872,9 @@
       </c>
       <c r="D18" s="4" t="inlineStr"/>
       <c r="E18" s="4" t="inlineStr"/>
-      <c r="F18" s="4" t="inlineStr"/>
+      <c r="F18" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="G18" s="4" t="inlineStr"/>
     </row>
     <row r="19">
@@ -860,7 +893,9 @@
       </c>
       <c r="D19" s="4" t="inlineStr"/>
       <c r="E19" s="4" t="inlineStr"/>
-      <c r="F19" s="4" t="inlineStr"/>
+      <c r="F19" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="G19" s="4" t="inlineStr"/>
     </row>
     <row r="20">
@@ -879,7 +914,9 @@
       </c>
       <c r="D20" s="4" t="inlineStr"/>
       <c r="E20" s="4" t="inlineStr"/>
-      <c r="F20" s="4" t="inlineStr"/>
+      <c r="F20" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="G20" s="4" t="inlineStr"/>
     </row>
     <row r="21">
@@ -898,7 +935,9 @@
       </c>
       <c r="D21" s="4" t="inlineStr"/>
       <c r="E21" s="4" t="inlineStr"/>
-      <c r="F21" s="4" t="inlineStr"/>
+      <c r="F21" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="G21" s="4" t="inlineStr"/>
     </row>
     <row r="22">
@@ -917,7 +956,9 @@
       </c>
       <c r="D22" s="4" t="inlineStr"/>
       <c r="E22" s="4" t="inlineStr"/>
-      <c r="F22" s="4" t="inlineStr"/>
+      <c r="F22" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="G22" s="4" t="inlineStr"/>
     </row>
     <row r="23">
@@ -936,7 +977,9 @@
       </c>
       <c r="D23" s="4" t="inlineStr"/>
       <c r="E23" s="4" t="inlineStr"/>
-      <c r="F23" s="4" t="inlineStr"/>
+      <c r="F23" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="G23" s="4" t="inlineStr"/>
     </row>
     <row r="24">
@@ -955,7 +998,9 @@
       </c>
       <c r="D24" s="4" t="inlineStr"/>
       <c r="E24" s="4" t="inlineStr"/>
-      <c r="F24" s="4" t="inlineStr"/>
+      <c r="F24" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="G24" s="4" t="inlineStr"/>
     </row>
     <row r="25">
@@ -974,7 +1019,9 @@
       </c>
       <c r="D25" s="4" t="inlineStr"/>
       <c r="E25" s="4" t="inlineStr"/>
-      <c r="F25" s="4" t="inlineStr"/>
+      <c r="F25" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="G25" s="4" t="inlineStr"/>
     </row>
     <row r="26">
@@ -993,7 +1040,9 @@
       </c>
       <c r="D26" s="4" t="inlineStr"/>
       <c r="E26" s="4" t="inlineStr"/>
-      <c r="F26" s="4" t="inlineStr"/>
+      <c r="F26" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="G26" s="4" t="inlineStr"/>
     </row>
     <row r="27">
@@ -1012,7 +1061,9 @@
       </c>
       <c r="D27" s="4" t="inlineStr"/>
       <c r="E27" s="4" t="inlineStr"/>
-      <c r="F27" s="4" t="inlineStr"/>
+      <c r="F27" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="G27" s="4" t="inlineStr"/>
     </row>
     <row r="28">
@@ -1031,7 +1082,9 @@
       </c>
       <c r="D28" s="4" t="inlineStr"/>
       <c r="E28" s="4" t="inlineStr"/>
-      <c r="F28" s="4" t="inlineStr"/>
+      <c r="F28" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="G28" s="4" t="inlineStr"/>
     </row>
     <row r="29">
@@ -1050,7 +1103,9 @@
       </c>
       <c r="D29" s="4" t="inlineStr"/>
       <c r="E29" s="4" t="inlineStr"/>
-      <c r="F29" s="4" t="inlineStr"/>
+      <c r="F29" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="G29" s="4" t="inlineStr"/>
     </row>
     <row r="30">
@@ -1069,7 +1124,9 @@
       </c>
       <c r="D30" s="4" t="inlineStr"/>
       <c r="E30" s="4" t="inlineStr"/>
-      <c r="F30" s="4" t="inlineStr"/>
+      <c r="F30" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="G30" s="4" t="inlineStr"/>
     </row>
     <row r="31">
@@ -1088,7 +1145,9 @@
       </c>
       <c r="D31" s="4" t="inlineStr"/>
       <c r="E31" s="4" t="inlineStr"/>
-      <c r="F31" s="4" t="inlineStr"/>
+      <c r="F31" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="G31" s="4" t="inlineStr"/>
     </row>
     <row r="32">
@@ -1103,7 +1162,9 @@
       <c r="C32" s="2" t="inlineStr"/>
       <c r="D32" s="4" t="inlineStr"/>
       <c r="E32" s="4" t="inlineStr"/>
-      <c r="F32" s="4" t="inlineStr"/>
+      <c r="F32" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="G32" s="4" t="inlineStr"/>
     </row>
     <row r="33">
@@ -1122,7 +1183,9 @@
       </c>
       <c r="D33" s="4" t="inlineStr"/>
       <c r="E33" s="4" t="inlineStr"/>
-      <c r="F33" s="4" t="inlineStr"/>
+      <c r="F33" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="G33" s="4" t="inlineStr"/>
     </row>
     <row r="34">
@@ -1141,7 +1204,9 @@
       </c>
       <c r="D34" s="4" t="inlineStr"/>
       <c r="E34" s="4" t="inlineStr"/>
-      <c r="F34" s="4" t="inlineStr"/>
+      <c r="F34" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="G34" s="4" t="inlineStr"/>
     </row>
     <row r="35">
@@ -1160,7 +1225,9 @@
       </c>
       <c r="D35" s="4" t="inlineStr"/>
       <c r="E35" s="4" t="inlineStr"/>
-      <c r="F35" s="4" t="inlineStr"/>
+      <c r="F35" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="G35" s="4" t="inlineStr"/>
     </row>
     <row r="36">
@@ -1179,7 +1246,9 @@
       </c>
       <c r="D36" s="4" t="inlineStr"/>
       <c r="E36" s="4" t="inlineStr"/>
-      <c r="F36" s="4" t="inlineStr"/>
+      <c r="F36" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="G36" s="4" t="inlineStr"/>
     </row>
     <row r="37">
@@ -1198,7 +1267,9 @@
       </c>
       <c r="D37" s="4" t="inlineStr"/>
       <c r="E37" s="4" t="inlineStr"/>
-      <c r="F37" s="4" t="inlineStr"/>
+      <c r="F37" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="G37" s="4" t="inlineStr"/>
     </row>
     <row r="38">
@@ -1213,7 +1284,9 @@
       <c r="C38" s="2" t="inlineStr"/>
       <c r="D38" s="4" t="inlineStr"/>
       <c r="E38" s="4" t="inlineStr"/>
-      <c r="F38" s="4" t="inlineStr"/>
+      <c r="F38" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="G38" s="4" t="inlineStr"/>
     </row>
     <row r="39">
@@ -1232,7 +1305,9 @@
       </c>
       <c r="D39" s="4" t="inlineStr"/>
       <c r="E39" s="4" t="inlineStr"/>
-      <c r="F39" s="4" t="inlineStr"/>
+      <c r="F39" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="G39" s="4" t="inlineStr"/>
     </row>
     <row r="40">
@@ -1251,7 +1326,9 @@
       </c>
       <c r="D40" s="4" t="inlineStr"/>
       <c r="E40" s="4" t="inlineStr"/>
-      <c r="F40" s="4" t="inlineStr"/>
+      <c r="F40" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="G40" s="4" t="inlineStr"/>
     </row>
     <row r="41">
@@ -1270,7 +1347,9 @@
       </c>
       <c r="D41" s="4" t="inlineStr"/>
       <c r="E41" s="4" t="inlineStr"/>
-      <c r="F41" s="4" t="inlineStr"/>
+      <c r="F41" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="G41" s="4" t="inlineStr"/>
     </row>
     <row r="42">
@@ -1289,7 +1368,9 @@
       </c>
       <c r="D42" s="4" t="inlineStr"/>
       <c r="E42" s="4" t="inlineStr"/>
-      <c r="F42" s="4" t="inlineStr"/>
+      <c r="F42" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="G42" s="4" t="inlineStr"/>
     </row>
     <row r="43">
@@ -1308,7 +1389,9 @@
       </c>
       <c r="D43" s="4" t="inlineStr"/>
       <c r="E43" s="4" t="inlineStr"/>
-      <c r="F43" s="4" t="inlineStr"/>
+      <c r="F43" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="G43" s="4" t="inlineStr"/>
     </row>
     <row r="44">
@@ -1327,7 +1410,9 @@
       </c>
       <c r="D44" s="4" t="inlineStr"/>
       <c r="E44" s="4" t="inlineStr"/>
-      <c r="F44" s="4" t="inlineStr"/>
+      <c r="F44" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="G44" s="4" t="inlineStr"/>
     </row>
     <row r="45">
@@ -1342,7 +1427,9 @@
       <c r="C45" s="2" t="inlineStr"/>
       <c r="D45" s="4" t="inlineStr"/>
       <c r="E45" s="4" t="inlineStr"/>
-      <c r="F45" s="4" t="inlineStr"/>
+      <c r="F45" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="G45" s="4" t="inlineStr"/>
     </row>
     <row r="46">
@@ -1357,7 +1444,9 @@
       <c r="C46" s="2" t="inlineStr"/>
       <c r="D46" s="4" t="inlineStr"/>
       <c r="E46" s="4" t="inlineStr"/>
-      <c r="F46" s="4" t="inlineStr"/>
+      <c r="F46" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="G46" s="4" t="inlineStr"/>
     </row>
     <row r="47">
@@ -1376,7 +1465,9 @@
       </c>
       <c r="D47" s="4" t="inlineStr"/>
       <c r="E47" s="4" t="inlineStr"/>
-      <c r="F47" s="4" t="inlineStr"/>
+      <c r="F47" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="G47" s="4" t="inlineStr"/>
     </row>
     <row r="48">
@@ -1395,7 +1486,9 @@
       </c>
       <c r="D48" s="4" t="inlineStr"/>
       <c r="E48" s="4" t="inlineStr"/>
-      <c r="F48" s="4" t="inlineStr"/>
+      <c r="F48" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="G48" s="4" t="inlineStr"/>
     </row>
     <row r="49">
@@ -1414,7 +1507,9 @@
       </c>
       <c r="D49" s="4" t="inlineStr"/>
       <c r="E49" s="4" t="inlineStr"/>
-      <c r="F49" s="4" t="inlineStr"/>
+      <c r="F49" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="G49" s="4" t="inlineStr"/>
     </row>
     <row r="50">
@@ -1433,7 +1528,9 @@
       </c>
       <c r="D50" s="4" t="inlineStr"/>
       <c r="E50" s="4" t="inlineStr"/>
-      <c r="F50" s="4" t="inlineStr"/>
+      <c r="F50" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="G50" s="4" t="inlineStr"/>
     </row>
     <row r="51">
@@ -1452,7 +1549,9 @@
       </c>
       <c r="D51" s="4" t="inlineStr"/>
       <c r="E51" s="4" t="inlineStr"/>
-      <c r="F51" s="4" t="inlineStr"/>
+      <c r="F51" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="G51" s="4" t="inlineStr"/>
     </row>
     <row r="52">
@@ -1471,7 +1570,9 @@
       </c>
       <c r="D52" s="4" t="inlineStr"/>
       <c r="E52" s="4" t="inlineStr"/>
-      <c r="F52" s="4" t="inlineStr"/>
+      <c r="F52" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="G52" s="4" t="inlineStr"/>
     </row>
     <row r="53">
@@ -1490,7 +1591,9 @@
       </c>
       <c r="D53" s="4" t="inlineStr"/>
       <c r="E53" s="4" t="inlineStr"/>
-      <c r="F53" s="4" t="inlineStr"/>
+      <c r="F53" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="G53" s="4" t="inlineStr"/>
     </row>
     <row r="54">
@@ -1509,7 +1612,9 @@
       </c>
       <c r="D54" s="4" t="inlineStr"/>
       <c r="E54" s="4" t="inlineStr"/>
-      <c r="F54" s="4" t="inlineStr"/>
+      <c r="F54" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="G54" s="4" t="inlineStr"/>
     </row>
     <row r="55">
@@ -1524,7 +1629,9 @@
       <c r="C55" s="2" t="inlineStr"/>
       <c r="D55" s="4" t="inlineStr"/>
       <c r="E55" s="4" t="inlineStr"/>
-      <c r="F55" s="4" t="inlineStr"/>
+      <c r="F55" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="G55" s="4" t="inlineStr"/>
     </row>
     <row r="56">
@@ -1543,7 +1650,9 @@
       </c>
       <c r="D56" s="4" t="inlineStr"/>
       <c r="E56" s="4" t="inlineStr"/>
-      <c r="F56" s="4" t="inlineStr"/>
+      <c r="F56" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="G56" s="4" t="inlineStr"/>
     </row>
     <row r="57">
@@ -1562,7 +1671,9 @@
       </c>
       <c r="D57" s="4" t="inlineStr"/>
       <c r="E57" s="4" t="inlineStr"/>
-      <c r="F57" s="4" t="inlineStr"/>
+      <c r="F57" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="G57" s="4" t="inlineStr"/>
     </row>
     <row r="58">
@@ -1581,7 +1692,9 @@
       </c>
       <c r="D58" s="4" t="inlineStr"/>
       <c r="E58" s="4" t="inlineStr"/>
-      <c r="F58" s="4" t="inlineStr"/>
+      <c r="F58" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="G58" s="4" t="inlineStr"/>
     </row>
     <row r="59">
@@ -1600,7 +1713,9 @@
       </c>
       <c r="D59" s="4" t="inlineStr"/>
       <c r="E59" s="4" t="inlineStr"/>
-      <c r="F59" s="4" t="inlineStr"/>
+      <c r="F59" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="G59" s="4" t="inlineStr"/>
     </row>
     <row r="60">
@@ -1619,7 +1734,9 @@
       </c>
       <c r="D60" s="4" t="inlineStr"/>
       <c r="E60" s="4" t="inlineStr"/>
-      <c r="F60" s="4" t="inlineStr"/>
+      <c r="F60" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="G60" s="4" t="inlineStr"/>
     </row>
     <row r="61">
@@ -1634,7 +1751,9 @@
       <c r="C61" s="2" t="inlineStr"/>
       <c r="D61" s="4" t="inlineStr"/>
       <c r="E61" s="4" t="inlineStr"/>
-      <c r="F61" s="4" t="inlineStr"/>
+      <c r="F61" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="G61" s="4" t="inlineStr"/>
     </row>
     <row r="62">
@@ -1653,7 +1772,9 @@
       </c>
       <c r="D62" s="7" t="inlineStr"/>
       <c r="E62" s="7" t="inlineStr"/>
-      <c r="F62" s="7" t="inlineStr"/>
+      <c r="F62" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G62" s="7" t="inlineStr"/>
     </row>
     <row r="63">
@@ -1672,7 +1793,9 @@
       </c>
       <c r="D63" s="7" t="inlineStr"/>
       <c r="E63" s="7" t="inlineStr"/>
-      <c r="F63" s="7" t="inlineStr"/>
+      <c r="F63" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G63" s="7" t="inlineStr"/>
     </row>
     <row r="64">
@@ -1691,7 +1814,9 @@
       </c>
       <c r="D64" s="7" t="inlineStr"/>
       <c r="E64" s="7" t="inlineStr"/>
-      <c r="F64" s="7" t="inlineStr"/>
+      <c r="F64" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G64" s="7" t="inlineStr"/>
     </row>
     <row r="65">
@@ -1710,7 +1835,9 @@
       </c>
       <c r="D65" s="7" t="inlineStr"/>
       <c r="E65" s="7" t="inlineStr"/>
-      <c r="F65" s="7" t="inlineStr"/>
+      <c r="F65" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G65" s="7" t="inlineStr"/>
     </row>
     <row r="66">
@@ -1729,7 +1856,9 @@
       </c>
       <c r="D66" s="7" t="inlineStr"/>
       <c r="E66" s="7" t="inlineStr"/>
-      <c r="F66" s="7" t="inlineStr"/>
+      <c r="F66" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G66" s="7" t="inlineStr"/>
     </row>
     <row r="67">
@@ -1748,7 +1877,9 @@
       </c>
       <c r="D67" s="7" t="inlineStr"/>
       <c r="E67" s="7" t="inlineStr"/>
-      <c r="F67" s="7" t="inlineStr"/>
+      <c r="F67" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G67" s="7" t="inlineStr"/>
     </row>
     <row r="68">
@@ -1767,7 +1898,9 @@
       </c>
       <c r="D68" s="7" t="inlineStr"/>
       <c r="E68" s="7" t="inlineStr"/>
-      <c r="F68" s="7" t="inlineStr"/>
+      <c r="F68" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G68" s="7" t="inlineStr"/>
     </row>
     <row r="69">
@@ -1786,7 +1919,9 @@
       </c>
       <c r="D69" s="7" t="inlineStr"/>
       <c r="E69" s="7" t="inlineStr"/>
-      <c r="F69" s="7" t="inlineStr"/>
+      <c r="F69" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G69" s="7" t="inlineStr"/>
     </row>
     <row r="70">
@@ -1805,7 +1940,9 @@
       </c>
       <c r="D70" s="7" t="inlineStr"/>
       <c r="E70" s="7" t="inlineStr"/>
-      <c r="F70" s="7" t="inlineStr"/>
+      <c r="F70" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G70" s="7" t="inlineStr"/>
     </row>
     <row r="71">
@@ -1824,7 +1961,9 @@
       </c>
       <c r="D71" s="7" t="inlineStr"/>
       <c r="E71" s="7" t="inlineStr"/>
-      <c r="F71" s="7" t="inlineStr"/>
+      <c r="F71" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G71" s="7" t="inlineStr"/>
     </row>
     <row r="72">
@@ -1843,7 +1982,9 @@
       </c>
       <c r="D72" s="7" t="inlineStr"/>
       <c r="E72" s="7" t="inlineStr"/>
-      <c r="F72" s="7" t="inlineStr"/>
+      <c r="F72" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G72" s="7" t="inlineStr"/>
     </row>
     <row r="73">
@@ -1862,7 +2003,9 @@
       </c>
       <c r="D73" s="7" t="inlineStr"/>
       <c r="E73" s="7" t="inlineStr"/>
-      <c r="F73" s="7" t="inlineStr"/>
+      <c r="F73" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G73" s="7" t="inlineStr"/>
     </row>
     <row r="74">
@@ -1881,7 +2024,9 @@
       </c>
       <c r="D74" s="7" t="inlineStr"/>
       <c r="E74" s="7" t="inlineStr"/>
-      <c r="F74" s="7" t="inlineStr"/>
+      <c r="F74" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G74" s="7" t="inlineStr"/>
     </row>
     <row r="75">
@@ -1900,7 +2045,9 @@
       </c>
       <c r="D75" s="7" t="inlineStr"/>
       <c r="E75" s="7" t="inlineStr"/>
-      <c r="F75" s="7" t="inlineStr"/>
+      <c r="F75" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G75" s="7" t="inlineStr"/>
     </row>
     <row r="76">
@@ -1919,7 +2066,9 @@
       </c>
       <c r="D76" s="7" t="inlineStr"/>
       <c r="E76" s="7" t="inlineStr"/>
-      <c r="F76" s="7" t="inlineStr"/>
+      <c r="F76" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G76" s="7" t="inlineStr"/>
     </row>
     <row r="77">
@@ -1938,7 +2087,9 @@
       </c>
       <c r="D77" s="7" t="inlineStr"/>
       <c r="E77" s="7" t="inlineStr"/>
-      <c r="F77" s="7" t="inlineStr"/>
+      <c r="F77" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G77" s="7" t="inlineStr"/>
     </row>
     <row r="78">
@@ -1957,7 +2108,9 @@
       </c>
       <c r="D78" s="7" t="inlineStr"/>
       <c r="E78" s="7" t="inlineStr"/>
-      <c r="F78" s="7" t="inlineStr"/>
+      <c r="F78" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G78" s="7" t="inlineStr"/>
     </row>
     <row r="79">
@@ -1976,7 +2129,9 @@
       </c>
       <c r="D79" s="7" t="inlineStr"/>
       <c r="E79" s="7" t="inlineStr"/>
-      <c r="F79" s="7" t="inlineStr"/>
+      <c r="F79" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G79" s="7" t="inlineStr"/>
     </row>
     <row r="80">
@@ -1991,7 +2146,9 @@
       <c r="C80" s="5" t="inlineStr"/>
       <c r="D80" s="7" t="inlineStr"/>
       <c r="E80" s="7" t="inlineStr"/>
-      <c r="F80" s="7" t="inlineStr"/>
+      <c r="F80" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G80" s="7" t="inlineStr"/>
     </row>
     <row r="81">
@@ -2006,7 +2163,9 @@
       <c r="C81" s="5" t="inlineStr"/>
       <c r="D81" s="7" t="inlineStr"/>
       <c r="E81" s="7" t="inlineStr"/>
-      <c r="F81" s="7" t="inlineStr"/>
+      <c r="F81" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G81" s="7" t="inlineStr"/>
     </row>
     <row r="82">
@@ -2025,7 +2184,9 @@
       </c>
       <c r="D82" s="7" t="inlineStr"/>
       <c r="E82" s="7" t="inlineStr"/>
-      <c r="F82" s="7" t="inlineStr"/>
+      <c r="F82" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G82" s="7" t="inlineStr"/>
     </row>
     <row r="83">
@@ -2044,7 +2205,9 @@
       </c>
       <c r="D83" s="7" t="inlineStr"/>
       <c r="E83" s="7" t="inlineStr"/>
-      <c r="F83" s="7" t="inlineStr"/>
+      <c r="F83" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G83" s="7" t="inlineStr"/>
     </row>
     <row r="84">
@@ -2063,7 +2226,9 @@
       </c>
       <c r="D84" s="7" t="inlineStr"/>
       <c r="E84" s="7" t="inlineStr"/>
-      <c r="F84" s="7" t="inlineStr"/>
+      <c r="F84" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G84" s="7" t="inlineStr"/>
     </row>
     <row r="85">
@@ -2082,7 +2247,9 @@
       </c>
       <c r="D85" s="7" t="inlineStr"/>
       <c r="E85" s="7" t="inlineStr"/>
-      <c r="F85" s="7" t="inlineStr"/>
+      <c r="F85" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G85" s="7" t="inlineStr"/>
     </row>
     <row r="86">
@@ -2101,7 +2268,9 @@
       </c>
       <c r="D86" s="7" t="inlineStr"/>
       <c r="E86" s="7" t="inlineStr"/>
-      <c r="F86" s="7" t="inlineStr"/>
+      <c r="F86" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G86" s="7" t="inlineStr"/>
     </row>
     <row r="87">
@@ -2120,7 +2289,9 @@
       </c>
       <c r="D87" s="7" t="inlineStr"/>
       <c r="E87" s="7" t="inlineStr"/>
-      <c r="F87" s="7" t="inlineStr"/>
+      <c r="F87" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G87" s="7" t="inlineStr"/>
     </row>
     <row r="88">
@@ -2139,7 +2310,9 @@
       </c>
       <c r="D88" s="7" t="inlineStr"/>
       <c r="E88" s="7" t="inlineStr"/>
-      <c r="F88" s="7" t="inlineStr"/>
+      <c r="F88" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G88" s="7" t="inlineStr"/>
     </row>
     <row r="89">
@@ -2158,7 +2331,9 @@
       </c>
       <c r="D89" s="7" t="inlineStr"/>
       <c r="E89" s="7" t="inlineStr"/>
-      <c r="F89" s="7" t="inlineStr"/>
+      <c r="F89" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G89" s="7" t="inlineStr"/>
     </row>
     <row r="90">
@@ -2177,7 +2352,9 @@
       </c>
       <c r="D90" s="7" t="inlineStr"/>
       <c r="E90" s="7" t="inlineStr"/>
-      <c r="F90" s="7" t="inlineStr"/>
+      <c r="F90" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G90" s="7" t="inlineStr"/>
     </row>
     <row r="91">
@@ -2196,7 +2373,9 @@
       </c>
       <c r="D91" s="7" t="inlineStr"/>
       <c r="E91" s="7" t="inlineStr"/>
-      <c r="F91" s="7" t="inlineStr"/>
+      <c r="F91" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G91" s="7" t="inlineStr"/>
     </row>
     <row r="92">
@@ -2211,7 +2390,9 @@
       <c r="C92" s="5" t="inlineStr"/>
       <c r="D92" s="7" t="inlineStr"/>
       <c r="E92" s="7" t="inlineStr"/>
-      <c r="F92" s="7" t="inlineStr"/>
+      <c r="F92" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G92" s="7" t="inlineStr"/>
     </row>
     <row r="93">
@@ -2230,7 +2411,9 @@
       </c>
       <c r="D93" s="7" t="inlineStr"/>
       <c r="E93" s="7" t="inlineStr"/>
-      <c r="F93" s="7" t="inlineStr"/>
+      <c r="F93" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G93" s="7" t="inlineStr"/>
     </row>
     <row r="94">
@@ -2249,7 +2432,9 @@
       </c>
       <c r="D94" s="7" t="inlineStr"/>
       <c r="E94" s="7" t="inlineStr"/>
-      <c r="F94" s="7" t="inlineStr"/>
+      <c r="F94" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G94" s="7" t="inlineStr"/>
     </row>
     <row r="95">
@@ -2268,7 +2453,9 @@
       </c>
       <c r="D95" s="7" t="inlineStr"/>
       <c r="E95" s="7" t="inlineStr"/>
-      <c r="F95" s="7" t="inlineStr"/>
+      <c r="F95" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G95" s="7" t="inlineStr"/>
     </row>
     <row r="96">
@@ -2287,7 +2474,9 @@
       </c>
       <c r="D96" s="7" t="inlineStr"/>
       <c r="E96" s="7" t="inlineStr"/>
-      <c r="F96" s="7" t="inlineStr"/>
+      <c r="F96" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G96" s="7" t="inlineStr"/>
     </row>
     <row r="97">
@@ -2306,7 +2495,9 @@
       </c>
       <c r="D97" s="7" t="inlineStr"/>
       <c r="E97" s="7" t="inlineStr"/>
-      <c r="F97" s="7" t="inlineStr"/>
+      <c r="F97" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G97" s="7" t="inlineStr"/>
     </row>
     <row r="98">
@@ -2325,7 +2516,9 @@
       </c>
       <c r="D98" s="7" t="inlineStr"/>
       <c r="E98" s="7" t="inlineStr"/>
-      <c r="F98" s="7" t="inlineStr"/>
+      <c r="F98" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G98" s="7" t="inlineStr"/>
     </row>
     <row r="99">
@@ -2344,7 +2537,9 @@
       </c>
       <c r="D99" s="7" t="inlineStr"/>
       <c r="E99" s="7" t="inlineStr"/>
-      <c r="F99" s="7" t="inlineStr"/>
+      <c r="F99" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G99" s="7" t="inlineStr"/>
     </row>
     <row r="100">
@@ -2363,7 +2558,9 @@
       </c>
       <c r="D100" s="7" t="inlineStr"/>
       <c r="E100" s="7" t="inlineStr"/>
-      <c r="F100" s="7" t="inlineStr"/>
+      <c r="F100" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G100" s="7" t="inlineStr"/>
     </row>
     <row r="101">
@@ -2382,7 +2579,9 @@
       </c>
       <c r="D101" s="7" t="inlineStr"/>
       <c r="E101" s="7" t="inlineStr"/>
-      <c r="F101" s="7" t="inlineStr"/>
+      <c r="F101" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G101" s="7" t="inlineStr"/>
     </row>
     <row r="102">
@@ -2401,7 +2600,9 @@
       </c>
       <c r="D102" s="7" t="inlineStr"/>
       <c r="E102" s="7" t="inlineStr"/>
-      <c r="F102" s="7" t="inlineStr"/>
+      <c r="F102" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G102" s="7" t="inlineStr"/>
     </row>
     <row r="103">
@@ -2420,7 +2621,9 @@
       </c>
       <c r="D103" s="7" t="inlineStr"/>
       <c r="E103" s="7" t="inlineStr"/>
-      <c r="F103" s="7" t="inlineStr"/>
+      <c r="F103" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G103" s="7" t="inlineStr"/>
     </row>
     <row r="104">
@@ -2439,7 +2642,9 @@
       </c>
       <c r="D104" s="7" t="inlineStr"/>
       <c r="E104" s="7" t="inlineStr"/>
-      <c r="F104" s="7" t="inlineStr"/>
+      <c r="F104" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G104" s="7" t="inlineStr"/>
     </row>
     <row r="105">
@@ -2458,7 +2663,9 @@
       </c>
       <c r="D105" s="7" t="inlineStr"/>
       <c r="E105" s="7" t="inlineStr"/>
-      <c r="F105" s="7" t="inlineStr"/>
+      <c r="F105" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G105" s="7" t="inlineStr"/>
     </row>
     <row r="106">
@@ -2477,7 +2684,9 @@
       </c>
       <c r="D106" s="7" t="inlineStr"/>
       <c r="E106" s="7" t="inlineStr"/>
-      <c r="F106" s="7" t="inlineStr"/>
+      <c r="F106" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G106" s="7" t="inlineStr"/>
     </row>
     <row r="107">
@@ -2496,7 +2705,9 @@
       </c>
       <c r="D107" s="7" t="inlineStr"/>
       <c r="E107" s="7" t="inlineStr"/>
-      <c r="F107" s="7" t="inlineStr"/>
+      <c r="F107" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G107" s="7" t="inlineStr"/>
     </row>
     <row r="108">
@@ -2515,7 +2726,9 @@
       </c>
       <c r="D108" s="7" t="inlineStr"/>
       <c r="E108" s="7" t="inlineStr"/>
-      <c r="F108" s="7" t="inlineStr"/>
+      <c r="F108" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G108" s="7" t="inlineStr"/>
     </row>
     <row r="109">
@@ -2534,7 +2747,9 @@
       </c>
       <c r="D109" s="7" t="inlineStr"/>
       <c r="E109" s="7" t="inlineStr"/>
-      <c r="F109" s="7" t="inlineStr"/>
+      <c r="F109" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G109" s="7" t="inlineStr"/>
     </row>
     <row r="110">
@@ -2553,7 +2768,9 @@
       </c>
       <c r="D110" s="7" t="inlineStr"/>
       <c r="E110" s="7" t="inlineStr"/>
-      <c r="F110" s="7" t="inlineStr"/>
+      <c r="F110" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G110" s="7" t="inlineStr"/>
     </row>
     <row r="111">
@@ -2572,7 +2789,9 @@
       </c>
       <c r="D111" s="7" t="inlineStr"/>
       <c r="E111" s="7" t="inlineStr"/>
-      <c r="F111" s="7" t="inlineStr"/>
+      <c r="F111" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G111" s="7" t="inlineStr"/>
     </row>
     <row r="112">
@@ -2591,7 +2810,9 @@
       </c>
       <c r="D112" s="7" t="inlineStr"/>
       <c r="E112" s="7" t="inlineStr"/>
-      <c r="F112" s="7" t="inlineStr"/>
+      <c r="F112" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G112" s="7" t="inlineStr"/>
     </row>
     <row r="113">
@@ -2610,7 +2831,9 @@
       </c>
       <c r="D113" s="7" t="inlineStr"/>
       <c r="E113" s="7" t="inlineStr"/>
-      <c r="F113" s="7" t="inlineStr"/>
+      <c r="F113" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G113" s="7" t="inlineStr"/>
     </row>
     <row r="114">
@@ -2629,7 +2852,9 @@
       </c>
       <c r="D114" s="7" t="inlineStr"/>
       <c r="E114" s="7" t="inlineStr"/>
-      <c r="F114" s="7" t="inlineStr"/>
+      <c r="F114" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G114" s="7" t="inlineStr"/>
     </row>
     <row r="115">
@@ -2648,7 +2873,9 @@
       </c>
       <c r="D115" s="7" t="inlineStr"/>
       <c r="E115" s="7" t="inlineStr"/>
-      <c r="F115" s="7" t="inlineStr"/>
+      <c r="F115" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G115" s="7" t="inlineStr"/>
     </row>
     <row r="116">
@@ -2663,7 +2890,9 @@
       <c r="C116" s="5" t="inlineStr"/>
       <c r="D116" s="7" t="inlineStr"/>
       <c r="E116" s="7" t="inlineStr"/>
-      <c r="F116" s="7" t="inlineStr"/>
+      <c r="F116" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G116" s="7" t="inlineStr"/>
     </row>
     <row r="117">
@@ -2682,7 +2911,9 @@
       </c>
       <c r="D117" s="7" t="inlineStr"/>
       <c r="E117" s="7" t="inlineStr"/>
-      <c r="F117" s="7" t="inlineStr"/>
+      <c r="F117" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G117" s="7" t="inlineStr"/>
     </row>
     <row r="118">
@@ -2701,7 +2932,9 @@
       </c>
       <c r="D118" s="7" t="inlineStr"/>
       <c r="E118" s="7" t="inlineStr"/>
-      <c r="F118" s="7" t="inlineStr"/>
+      <c r="F118" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G118" s="7" t="inlineStr"/>
     </row>
     <row r="119">
@@ -2720,7 +2953,9 @@
       </c>
       <c r="D119" s="7" t="inlineStr"/>
       <c r="E119" s="7" t="inlineStr"/>
-      <c r="F119" s="7" t="inlineStr"/>
+      <c r="F119" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G119" s="7" t="inlineStr"/>
     </row>
     <row r="120">
@@ -2739,7 +2974,9 @@
       </c>
       <c r="D120" s="7" t="inlineStr"/>
       <c r="E120" s="7" t="inlineStr"/>
-      <c r="F120" s="7" t="inlineStr"/>
+      <c r="F120" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G120" s="7" t="inlineStr"/>
     </row>
     <row r="121">
@@ -2758,7 +2995,9 @@
       </c>
       <c r="D121" s="7" t="inlineStr"/>
       <c r="E121" s="7" t="inlineStr"/>
-      <c r="F121" s="7" t="inlineStr"/>
+      <c r="F121" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G121" s="7" t="inlineStr"/>
     </row>
     <row r="122">
@@ -2777,7 +3016,9 @@
       </c>
       <c r="D122" s="7" t="inlineStr"/>
       <c r="E122" s="7" t="inlineStr"/>
-      <c r="F122" s="7" t="inlineStr"/>
+      <c r="F122" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G122" s="7" t="inlineStr"/>
     </row>
     <row r="123">
@@ -2796,7 +3037,9 @@
       </c>
       <c r="D123" s="7" t="inlineStr"/>
       <c r="E123" s="7" t="inlineStr"/>
-      <c r="F123" s="7" t="inlineStr"/>
+      <c r="F123" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G123" s="7" t="inlineStr"/>
     </row>
     <row r="124">
@@ -2815,7 +3058,9 @@
       </c>
       <c r="D124" s="7" t="inlineStr"/>
       <c r="E124" s="7" t="inlineStr"/>
-      <c r="F124" s="7" t="inlineStr"/>
+      <c r="F124" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G124" s="7" t="inlineStr"/>
     </row>
     <row r="125">
@@ -2830,7 +3075,9 @@
       <c r="C125" s="5" t="inlineStr"/>
       <c r="D125" s="7" t="inlineStr"/>
       <c r="E125" s="7" t="inlineStr"/>
-      <c r="F125" s="7" t="inlineStr"/>
+      <c r="F125" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G125" s="7" t="inlineStr"/>
     </row>
     <row r="126">
@@ -2849,7 +3096,9 @@
       </c>
       <c r="D126" s="7" t="inlineStr"/>
       <c r="E126" s="7" t="inlineStr"/>
-      <c r="F126" s="7" t="inlineStr"/>
+      <c r="F126" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G126" s="7" t="inlineStr"/>
     </row>
     <row r="127">
@@ -2868,7 +3117,9 @@
       </c>
       <c r="D127" s="7" t="inlineStr"/>
       <c r="E127" s="7" t="inlineStr"/>
-      <c r="F127" s="7" t="inlineStr"/>
+      <c r="F127" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G127" s="7" t="inlineStr"/>
     </row>
     <row r="128">
@@ -2887,7 +3138,9 @@
       </c>
       <c r="D128" s="7" t="inlineStr"/>
       <c r="E128" s="7" t="inlineStr"/>
-      <c r="F128" s="7" t="inlineStr"/>
+      <c r="F128" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G128" s="7" t="inlineStr"/>
     </row>
     <row r="129">
@@ -2906,7 +3159,9 @@
       </c>
       <c r="D129" s="7" t="inlineStr"/>
       <c r="E129" s="7" t="inlineStr"/>
-      <c r="F129" s="7" t="inlineStr"/>
+      <c r="F129" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G129" s="7" t="inlineStr"/>
     </row>
     <row r="130">
@@ -2925,7 +3180,9 @@
       </c>
       <c r="D130" s="7" t="inlineStr"/>
       <c r="E130" s="7" t="inlineStr"/>
-      <c r="F130" s="7" t="inlineStr"/>
+      <c r="F130" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G130" s="7" t="inlineStr"/>
     </row>
     <row r="131">
@@ -2944,7 +3201,9 @@
       </c>
       <c r="D131" s="7" t="inlineStr"/>
       <c r="E131" s="7" t="inlineStr"/>
-      <c r="F131" s="7" t="inlineStr"/>
+      <c r="F131" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G131" s="7" t="inlineStr"/>
     </row>
     <row r="132">
@@ -2963,7 +3222,9 @@
       </c>
       <c r="D132" s="7" t="inlineStr"/>
       <c r="E132" s="7" t="inlineStr"/>
-      <c r="F132" s="7" t="inlineStr"/>
+      <c r="F132" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G132" s="7" t="inlineStr"/>
     </row>
     <row r="133">
@@ -2982,7 +3243,9 @@
       </c>
       <c r="D133" s="7" t="inlineStr"/>
       <c r="E133" s="7" t="inlineStr"/>
-      <c r="F133" s="7" t="inlineStr"/>
+      <c r="F133" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G133" s="7" t="inlineStr"/>
     </row>
     <row r="134">
@@ -3001,7 +3264,9 @@
       </c>
       <c r="D134" s="7" t="inlineStr"/>
       <c r="E134" s="7" t="inlineStr"/>
-      <c r="F134" s="7" t="inlineStr"/>
+      <c r="F134" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G134" s="7" t="inlineStr"/>
     </row>
     <row r="135">
@@ -3020,7 +3285,9 @@
       </c>
       <c r="D135" s="7" t="inlineStr"/>
       <c r="E135" s="7" t="inlineStr"/>
-      <c r="F135" s="7" t="inlineStr"/>
+      <c r="F135" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G135" s="7" t="inlineStr"/>
     </row>
     <row r="136">
@@ -3039,7 +3306,9 @@
       </c>
       <c r="D136" s="7" t="inlineStr"/>
       <c r="E136" s="7" t="inlineStr"/>
-      <c r="F136" s="7" t="inlineStr"/>
+      <c r="F136" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G136" s="7" t="inlineStr"/>
     </row>
     <row r="137">
@@ -3058,7 +3327,9 @@
       </c>
       <c r="D137" s="7" t="inlineStr"/>
       <c r="E137" s="7" t="inlineStr"/>
-      <c r="F137" s="7" t="inlineStr"/>
+      <c r="F137" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G137" s="7" t="inlineStr"/>
     </row>
     <row r="138">
@@ -3077,7 +3348,9 @@
       </c>
       <c r="D138" s="7" t="inlineStr"/>
       <c r="E138" s="7" t="inlineStr"/>
-      <c r="F138" s="7" t="inlineStr"/>
+      <c r="F138" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G138" s="7" t="inlineStr"/>
     </row>
     <row r="139">
@@ -3096,7 +3369,9 @@
       </c>
       <c r="D139" s="7" t="inlineStr"/>
       <c r="E139" s="7" t="inlineStr"/>
-      <c r="F139" s="7" t="inlineStr"/>
+      <c r="F139" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G139" s="7" t="inlineStr"/>
     </row>
     <row r="140">
@@ -3115,7 +3390,9 @@
       </c>
       <c r="D140" s="7" t="inlineStr"/>
       <c r="E140" s="7" t="inlineStr"/>
-      <c r="F140" s="7" t="inlineStr"/>
+      <c r="F140" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G140" s="7" t="inlineStr"/>
     </row>
     <row r="141">
@@ -3134,7 +3411,9 @@
       </c>
       <c r="D141" s="7" t="inlineStr"/>
       <c r="E141" s="7" t="inlineStr"/>
-      <c r="F141" s="7" t="inlineStr"/>
+      <c r="F141" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G141" s="7" t="inlineStr"/>
     </row>
     <row r="142">
@@ -3153,7 +3432,9 @@
       </c>
       <c r="D142" s="7" t="inlineStr"/>
       <c r="E142" s="7" t="inlineStr"/>
-      <c r="F142" s="7" t="inlineStr"/>
+      <c r="F142" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G142" s="7" t="inlineStr"/>
     </row>
     <row r="143">
@@ -3172,7 +3453,9 @@
       </c>
       <c r="D143" s="7" t="inlineStr"/>
       <c r="E143" s="7" t="inlineStr"/>
-      <c r="F143" s="7" t="inlineStr"/>
+      <c r="F143" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G143" s="7" t="inlineStr"/>
     </row>
     <row r="144">
@@ -3191,7 +3474,9 @@
       </c>
       <c r="D144" s="7" t="inlineStr"/>
       <c r="E144" s="7" t="inlineStr"/>
-      <c r="F144" s="7" t="inlineStr"/>
+      <c r="F144" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G144" s="7" t="inlineStr"/>
     </row>
     <row r="145">
@@ -3210,7 +3495,9 @@
       </c>
       <c r="D145" s="7" t="inlineStr"/>
       <c r="E145" s="7" t="inlineStr"/>
-      <c r="F145" s="7" t="inlineStr"/>
+      <c r="F145" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G145" s="7" t="inlineStr"/>
     </row>
     <row r="146">
@@ -3229,7 +3516,9 @@
       </c>
       <c r="D146" s="7" t="inlineStr"/>
       <c r="E146" s="7" t="inlineStr"/>
-      <c r="F146" s="7" t="inlineStr"/>
+      <c r="F146" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G146" s="7" t="inlineStr"/>
     </row>
     <row r="147">
@@ -3248,7 +3537,9 @@
       </c>
       <c r="D147" s="7" t="inlineStr"/>
       <c r="E147" s="7" t="inlineStr"/>
-      <c r="F147" s="7" t="inlineStr"/>
+      <c r="F147" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G147" s="7" t="inlineStr"/>
     </row>
     <row r="148">
@@ -3267,7 +3558,9 @@
       </c>
       <c r="D148" s="7" t="inlineStr"/>
       <c r="E148" s="7" t="inlineStr"/>
-      <c r="F148" s="7" t="inlineStr"/>
+      <c r="F148" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G148" s="7" t="inlineStr"/>
     </row>
     <row r="149">
@@ -3286,7 +3579,9 @@
       </c>
       <c r="D149" s="7" t="inlineStr"/>
       <c r="E149" s="7" t="inlineStr"/>
-      <c r="F149" s="7" t="inlineStr"/>
+      <c r="F149" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G149" s="7" t="inlineStr"/>
     </row>
     <row r="150">
@@ -3305,7 +3600,9 @@
       </c>
       <c r="D150" s="7" t="inlineStr"/>
       <c r="E150" s="7" t="inlineStr"/>
-      <c r="F150" s="7" t="inlineStr"/>
+      <c r="F150" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G150" s="7" t="inlineStr"/>
     </row>
     <row r="151">
@@ -3324,7 +3621,9 @@
       </c>
       <c r="D151" s="7" t="inlineStr"/>
       <c r="E151" s="7" t="inlineStr"/>
-      <c r="F151" s="7" t="inlineStr"/>
+      <c r="F151" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G151" s="7" t="inlineStr"/>
     </row>
     <row r="152">
@@ -3343,7 +3642,9 @@
       </c>
       <c r="D152" s="7" t="inlineStr"/>
       <c r="E152" s="7" t="inlineStr"/>
-      <c r="F152" s="7" t="inlineStr"/>
+      <c r="F152" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G152" s="7" t="inlineStr"/>
     </row>
     <row r="153">
@@ -3362,7 +3663,9 @@
       </c>
       <c r="D153" s="7" t="inlineStr"/>
       <c r="E153" s="7" t="inlineStr"/>
-      <c r="F153" s="7" t="inlineStr"/>
+      <c r="F153" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G153" s="7" t="inlineStr"/>
     </row>
     <row r="154">
@@ -3381,7 +3684,9 @@
       </c>
       <c r="D154" s="7" t="inlineStr"/>
       <c r="E154" s="7" t="inlineStr"/>
-      <c r="F154" s="7" t="inlineStr"/>
+      <c r="F154" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G154" s="7" t="inlineStr"/>
     </row>
     <row r="155">
@@ -3400,7 +3705,9 @@
       </c>
       <c r="D155" s="7" t="inlineStr"/>
       <c r="E155" s="7" t="inlineStr"/>
-      <c r="F155" s="7" t="inlineStr"/>
+      <c r="F155" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G155" s="7" t="inlineStr"/>
     </row>
     <row r="156">
@@ -3419,7 +3726,9 @@
       </c>
       <c r="D156" s="7" t="inlineStr"/>
       <c r="E156" s="7" t="inlineStr"/>
-      <c r="F156" s="7" t="inlineStr"/>
+      <c r="F156" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G156" s="7" t="inlineStr"/>
     </row>
     <row r="157">
@@ -3438,7 +3747,9 @@
       </c>
       <c r="D157" s="7" t="inlineStr"/>
       <c r="E157" s="7" t="inlineStr"/>
-      <c r="F157" s="7" t="inlineStr"/>
+      <c r="F157" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G157" s="7" t="inlineStr"/>
     </row>
     <row r="158">
@@ -3457,7 +3768,9 @@
       </c>
       <c r="D158" s="7" t="inlineStr"/>
       <c r="E158" s="7" t="inlineStr"/>
-      <c r="F158" s="7" t="inlineStr"/>
+      <c r="F158" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G158" s="7" t="inlineStr"/>
     </row>
     <row r="159">
@@ -3476,7 +3789,9 @@
       </c>
       <c r="D159" s="7" t="inlineStr"/>
       <c r="E159" s="7" t="inlineStr"/>
-      <c r="F159" s="7" t="inlineStr"/>
+      <c r="F159" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G159" s="7" t="inlineStr"/>
     </row>
     <row r="160">
@@ -3495,7 +3810,9 @@
       </c>
       <c r="D160" s="7" t="inlineStr"/>
       <c r="E160" s="7" t="inlineStr"/>
-      <c r="F160" s="7" t="inlineStr"/>
+      <c r="F160" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G160" s="7" t="inlineStr"/>
     </row>
     <row r="161">
@@ -3514,7 +3831,9 @@
       </c>
       <c r="D161" s="7" t="inlineStr"/>
       <c r="E161" s="7" t="inlineStr"/>
-      <c r="F161" s="7" t="inlineStr"/>
+      <c r="F161" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G161" s="7" t="inlineStr"/>
     </row>
     <row r="162">
@@ -3533,7 +3852,9 @@
       </c>
       <c r="D162" s="7" t="inlineStr"/>
       <c r="E162" s="7" t="inlineStr"/>
-      <c r="F162" s="7" t="inlineStr"/>
+      <c r="F162" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G162" s="7" t="inlineStr"/>
     </row>
     <row r="163">
@@ -3552,7 +3873,9 @@
       </c>
       <c r="D163" s="7" t="inlineStr"/>
       <c r="E163" s="7" t="inlineStr"/>
-      <c r="F163" s="7" t="inlineStr"/>
+      <c r="F163" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G163" s="7" t="inlineStr"/>
     </row>
     <row r="164">
@@ -3571,7 +3894,9 @@
       </c>
       <c r="D164" s="7" t="inlineStr"/>
       <c r="E164" s="7" t="inlineStr"/>
-      <c r="F164" s="7" t="inlineStr"/>
+      <c r="F164" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G164" s="7" t="inlineStr"/>
     </row>
     <row r="165">
@@ -3586,7 +3911,9 @@
       <c r="C165" s="5" t="inlineStr"/>
       <c r="D165" s="7" t="inlineStr"/>
       <c r="E165" s="7" t="inlineStr"/>
-      <c r="F165" s="7" t="inlineStr"/>
+      <c r="F165" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G165" s="7" t="inlineStr"/>
     </row>
     <row r="166">
@@ -3605,7 +3932,9 @@
       </c>
       <c r="D166" s="7" t="inlineStr"/>
       <c r="E166" s="7" t="inlineStr"/>
-      <c r="F166" s="7" t="inlineStr"/>
+      <c r="F166" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G166" s="7" t="inlineStr"/>
     </row>
     <row r="167">
@@ -3624,7 +3953,9 @@
       </c>
       <c r="D167" s="7" t="inlineStr"/>
       <c r="E167" s="7" t="inlineStr"/>
-      <c r="F167" s="7" t="inlineStr"/>
+      <c r="F167" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G167" s="7" t="inlineStr"/>
     </row>
     <row r="168">
@@ -3643,7 +3974,9 @@
       </c>
       <c r="D168" s="7" t="inlineStr"/>
       <c r="E168" s="7" t="inlineStr"/>
-      <c r="F168" s="7" t="inlineStr"/>
+      <c r="F168" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G168" s="7" t="inlineStr"/>
     </row>
     <row r="169">
@@ -3662,7 +3995,9 @@
       </c>
       <c r="D169" s="7" t="inlineStr"/>
       <c r="E169" s="7" t="inlineStr"/>
-      <c r="F169" s="7" t="inlineStr"/>
+      <c r="F169" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G169" s="7" t="inlineStr"/>
     </row>
     <row r="170">
@@ -3681,7 +4016,9 @@
       </c>
       <c r="D170" s="7" t="inlineStr"/>
       <c r="E170" s="7" t="inlineStr"/>
-      <c r="F170" s="7" t="inlineStr"/>
+      <c r="F170" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G170" s="7" t="inlineStr"/>
     </row>
     <row r="171">
@@ -3700,7 +4037,9 @@
       </c>
       <c r="D171" s="7" t="inlineStr"/>
       <c r="E171" s="7" t="inlineStr"/>
-      <c r="F171" s="7" t="inlineStr"/>
+      <c r="F171" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G171" s="7" t="inlineStr"/>
     </row>
     <row r="172">
@@ -3719,7 +4058,9 @@
       </c>
       <c r="D172" s="7" t="inlineStr"/>
       <c r="E172" s="7" t="inlineStr"/>
-      <c r="F172" s="7" t="inlineStr"/>
+      <c r="F172" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G172" s="7" t="inlineStr"/>
     </row>
     <row r="173">
@@ -3738,7 +4079,9 @@
       </c>
       <c r="D173" s="7" t="inlineStr"/>
       <c r="E173" s="7" t="inlineStr"/>
-      <c r="F173" s="7" t="inlineStr"/>
+      <c r="F173" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G173" s="7" t="inlineStr"/>
     </row>
     <row r="174">
@@ -3757,7 +4100,9 @@
       </c>
       <c r="D174" s="7" t="inlineStr"/>
       <c r="E174" s="7" t="inlineStr"/>
-      <c r="F174" s="7" t="inlineStr"/>
+      <c r="F174" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G174" s="7" t="inlineStr"/>
     </row>
     <row r="175">
@@ -3776,7 +4121,9 @@
       </c>
       <c r="D175" s="7" t="inlineStr"/>
       <c r="E175" s="7" t="inlineStr"/>
-      <c r="F175" s="7" t="inlineStr"/>
+      <c r="F175" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G175" s="7" t="inlineStr"/>
     </row>
     <row r="176">
@@ -3795,7 +4142,9 @@
       </c>
       <c r="D176" s="7" t="inlineStr"/>
       <c r="E176" s="7" t="inlineStr"/>
-      <c r="F176" s="7" t="inlineStr"/>
+      <c r="F176" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G176" s="7" t="inlineStr"/>
     </row>
     <row r="177">
@@ -3814,7 +4163,9 @@
       </c>
       <c r="D177" s="7" t="inlineStr"/>
       <c r="E177" s="7" t="inlineStr"/>
-      <c r="F177" s="7" t="inlineStr"/>
+      <c r="F177" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G177" s="7" t="inlineStr"/>
     </row>
     <row r="178">
@@ -3833,7 +4184,9 @@
       </c>
       <c r="D178" s="7" t="inlineStr"/>
       <c r="E178" s="7" t="inlineStr"/>
-      <c r="F178" s="7" t="inlineStr"/>
+      <c r="F178" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G178" s="7" t="inlineStr"/>
     </row>
     <row r="179">
@@ -3852,7 +4205,9 @@
       </c>
       <c r="D179" s="7" t="inlineStr"/>
       <c r="E179" s="7" t="inlineStr"/>
-      <c r="F179" s="7" t="inlineStr"/>
+      <c r="F179" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G179" s="7" t="inlineStr"/>
     </row>
     <row r="180">
@@ -3867,7 +4222,9 @@
       <c r="C180" s="5" t="inlineStr"/>
       <c r="D180" s="7" t="inlineStr"/>
       <c r="E180" s="7" t="inlineStr"/>
-      <c r="F180" s="7" t="inlineStr"/>
+      <c r="F180" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G180" s="7" t="inlineStr"/>
     </row>
     <row r="181">
@@ -3886,7 +4243,9 @@
       </c>
       <c r="D181" s="7" t="inlineStr"/>
       <c r="E181" s="7" t="inlineStr"/>
-      <c r="F181" s="7" t="inlineStr"/>
+      <c r="F181" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G181" s="7" t="inlineStr"/>
     </row>
     <row r="182">
@@ -3905,7 +4264,9 @@
       </c>
       <c r="D182" s="7" t="inlineStr"/>
       <c r="E182" s="7" t="inlineStr"/>
-      <c r="F182" s="7" t="inlineStr"/>
+      <c r="F182" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G182" s="7" t="inlineStr"/>
     </row>
     <row r="183">
@@ -3924,7 +4285,9 @@
       </c>
       <c r="D183" s="7" t="inlineStr"/>
       <c r="E183" s="7" t="inlineStr"/>
-      <c r="F183" s="7" t="inlineStr"/>
+      <c r="F183" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G183" s="7" t="inlineStr"/>
     </row>
     <row r="184">
@@ -3943,7 +4306,9 @@
       </c>
       <c r="D184" s="7" t="inlineStr"/>
       <c r="E184" s="7" t="inlineStr"/>
-      <c r="F184" s="7" t="inlineStr"/>
+      <c r="F184" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G184" s="7" t="inlineStr"/>
     </row>
     <row r="185">
@@ -3962,7 +4327,9 @@
       </c>
       <c r="D185" s="7" t="inlineStr"/>
       <c r="E185" s="7" t="inlineStr"/>
-      <c r="F185" s="7" t="inlineStr"/>
+      <c r="F185" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G185" s="7" t="inlineStr"/>
     </row>
     <row r="186">
@@ -3981,7 +4348,9 @@
       </c>
       <c r="D186" s="7" t="inlineStr"/>
       <c r="E186" s="7" t="inlineStr"/>
-      <c r="F186" s="7" t="inlineStr"/>
+      <c r="F186" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G186" s="7" t="inlineStr"/>
     </row>
     <row r="187">
@@ -3996,7 +4365,9 @@
       <c r="C187" s="5" t="inlineStr"/>
       <c r="D187" s="7" t="inlineStr"/>
       <c r="E187" s="7" t="inlineStr"/>
-      <c r="F187" s="7" t="inlineStr"/>
+      <c r="F187" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G187" s="7" t="inlineStr"/>
     </row>
     <row r="188">
@@ -4015,7 +4386,9 @@
       </c>
       <c r="D188" s="7" t="inlineStr"/>
       <c r="E188" s="7" t="inlineStr"/>
-      <c r="F188" s="7" t="inlineStr"/>
+      <c r="F188" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G188" s="7" t="inlineStr"/>
     </row>
     <row r="189">
@@ -4034,7 +4407,9 @@
       </c>
       <c r="D189" s="7" t="inlineStr"/>
       <c r="E189" s="7" t="inlineStr"/>
-      <c r="F189" s="7" t="inlineStr"/>
+      <c r="F189" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G189" s="7" t="inlineStr"/>
     </row>
     <row r="190">
@@ -4053,7 +4428,9 @@
       </c>
       <c r="D190" s="7" t="inlineStr"/>
       <c r="E190" s="7" t="inlineStr"/>
-      <c r="F190" s="7" t="inlineStr"/>
+      <c r="F190" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G190" s="7" t="inlineStr"/>
     </row>
     <row r="191">
@@ -4072,7 +4449,9 @@
       </c>
       <c r="D191" s="7" t="inlineStr"/>
       <c r="E191" s="7" t="inlineStr"/>
-      <c r="F191" s="7" t="inlineStr"/>
+      <c r="F191" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G191" s="7" t="inlineStr"/>
     </row>
     <row r="192">
@@ -4091,7 +4470,9 @@
       </c>
       <c r="D192" s="7" t="inlineStr"/>
       <c r="E192" s="7" t="inlineStr"/>
-      <c r="F192" s="7" t="inlineStr"/>
+      <c r="F192" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G192" s="7" t="inlineStr"/>
     </row>
     <row r="193">
@@ -4110,7 +4491,9 @@
       </c>
       <c r="D193" s="7" t="inlineStr"/>
       <c r="E193" s="7" t="inlineStr"/>
-      <c r="F193" s="7" t="inlineStr"/>
+      <c r="F193" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G193" s="7" t="inlineStr"/>
     </row>
     <row r="194">
@@ -4129,7 +4512,9 @@
       </c>
       <c r="D194" s="7" t="inlineStr"/>
       <c r="E194" s="7" t="inlineStr"/>
-      <c r="F194" s="7" t="inlineStr"/>
+      <c r="F194" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G194" s="7" t="inlineStr"/>
     </row>
     <row r="195">
@@ -4148,7 +4533,9 @@
       </c>
       <c r="D195" s="7" t="inlineStr"/>
       <c r="E195" s="7" t="inlineStr"/>
-      <c r="F195" s="7" t="inlineStr"/>
+      <c r="F195" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G195" s="7" t="inlineStr"/>
     </row>
     <row r="196">
@@ -4167,7 +4554,9 @@
       </c>
       <c r="D196" s="7" t="inlineStr"/>
       <c r="E196" s="7" t="inlineStr"/>
-      <c r="F196" s="7" t="inlineStr"/>
+      <c r="F196" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G196" s="7" t="inlineStr"/>
     </row>
     <row r="197">
@@ -4186,7 +4575,9 @@
       </c>
       <c r="D197" s="7" t="inlineStr"/>
       <c r="E197" s="7" t="inlineStr"/>
-      <c r="F197" s="7" t="inlineStr"/>
+      <c r="F197" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G197" s="7" t="inlineStr"/>
     </row>
     <row r="198">
@@ -4205,7 +4596,9 @@
       </c>
       <c r="D198" s="7" t="inlineStr"/>
       <c r="E198" s="7" t="inlineStr"/>
-      <c r="F198" s="7" t="inlineStr"/>
+      <c r="F198" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G198" s="7" t="inlineStr"/>
     </row>
     <row r="199">
@@ -4224,7 +4617,9 @@
       </c>
       <c r="D199" s="7" t="inlineStr"/>
       <c r="E199" s="7" t="inlineStr"/>
-      <c r="F199" s="7" t="inlineStr"/>
+      <c r="F199" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G199" s="7" t="inlineStr"/>
     </row>
     <row r="200">
@@ -4243,7 +4638,9 @@
       </c>
       <c r="D200" s="7" t="inlineStr"/>
       <c r="E200" s="7" t="inlineStr"/>
-      <c r="F200" s="7" t="inlineStr"/>
+      <c r="F200" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G200" s="7" t="inlineStr"/>
     </row>
     <row r="201">
@@ -4262,7 +4659,9 @@
       </c>
       <c r="D201" s="7" t="inlineStr"/>
       <c r="E201" s="7" t="inlineStr"/>
-      <c r="F201" s="7" t="inlineStr"/>
+      <c r="F201" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G201" s="7" t="inlineStr"/>
     </row>
     <row r="202">
@@ -4281,7 +4680,9 @@
       </c>
       <c r="D202" s="7" t="inlineStr"/>
       <c r="E202" s="7" t="inlineStr"/>
-      <c r="F202" s="7" t="inlineStr"/>
+      <c r="F202" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G202" s="7" t="inlineStr"/>
     </row>
     <row r="203">
@@ -4300,7 +4701,9 @@
       </c>
       <c r="D203" s="7" t="inlineStr"/>
       <c r="E203" s="7" t="inlineStr"/>
-      <c r="F203" s="7" t="inlineStr"/>
+      <c r="F203" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G203" s="7" t="inlineStr"/>
     </row>
     <row r="204">
@@ -4319,7 +4722,9 @@
       </c>
       <c r="D204" s="7" t="inlineStr"/>
       <c r="E204" s="7" t="inlineStr"/>
-      <c r="F204" s="7" t="inlineStr"/>
+      <c r="F204" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G204" s="7" t="inlineStr"/>
     </row>
     <row r="205">
@@ -4338,7 +4743,9 @@
       </c>
       <c r="D205" s="7" t="inlineStr"/>
       <c r="E205" s="7" t="inlineStr"/>
-      <c r="F205" s="7" t="inlineStr"/>
+      <c r="F205" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G205" s="7" t="inlineStr"/>
     </row>
     <row r="206">
@@ -4357,7 +4764,9 @@
       </c>
       <c r="D206" s="7" t="inlineStr"/>
       <c r="E206" s="7" t="inlineStr"/>
-      <c r="F206" s="7" t="inlineStr"/>
+      <c r="F206" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G206" s="7" t="inlineStr"/>
     </row>
     <row r="207">
@@ -4376,7 +4785,9 @@
       </c>
       <c r="D207" s="7" t="inlineStr"/>
       <c r="E207" s="7" t="inlineStr"/>
-      <c r="F207" s="7" t="inlineStr"/>
+      <c r="F207" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G207" s="7" t="inlineStr"/>
     </row>
     <row r="208">
@@ -4395,7 +4806,9 @@
       </c>
       <c r="D208" s="7" t="inlineStr"/>
       <c r="E208" s="7" t="inlineStr"/>
-      <c r="F208" s="7" t="inlineStr"/>
+      <c r="F208" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G208" s="7" t="inlineStr"/>
     </row>
     <row r="209">
@@ -4414,7 +4827,9 @@
       </c>
       <c r="D209" s="7" t="inlineStr"/>
       <c r="E209" s="7" t="inlineStr"/>
-      <c r="F209" s="7" t="inlineStr"/>
+      <c r="F209" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G209" s="7" t="inlineStr"/>
     </row>
     <row r="210">
@@ -4433,7 +4848,9 @@
       </c>
       <c r="D210" s="7" t="inlineStr"/>
       <c r="E210" s="7" t="inlineStr"/>
-      <c r="F210" s="7" t="inlineStr"/>
+      <c r="F210" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G210" s="7" t="inlineStr"/>
     </row>
     <row r="211">
@@ -4452,7 +4869,9 @@
       </c>
       <c r="D211" s="7" t="inlineStr"/>
       <c r="E211" s="7" t="inlineStr"/>
-      <c r="F211" s="7" t="inlineStr"/>
+      <c r="F211" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G211" s="7" t="inlineStr"/>
     </row>
     <row r="212">
@@ -4471,7 +4890,9 @@
       </c>
       <c r="D212" s="7" t="inlineStr"/>
       <c r="E212" s="7" t="inlineStr"/>
-      <c r="F212" s="7" t="inlineStr"/>
+      <c r="F212" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G212" s="7" t="inlineStr"/>
     </row>
     <row r="213">
@@ -4486,7 +4907,9 @@
       <c r="C213" s="5" t="inlineStr"/>
       <c r="D213" s="7" t="inlineStr"/>
       <c r="E213" s="7" t="inlineStr"/>
-      <c r="F213" s="7" t="inlineStr"/>
+      <c r="F213" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G213" s="7" t="inlineStr"/>
     </row>
     <row r="214">
@@ -4505,7 +4928,9 @@
       </c>
       <c r="D214" s="7" t="inlineStr"/>
       <c r="E214" s="7" t="inlineStr"/>
-      <c r="F214" s="7" t="inlineStr"/>
+      <c r="F214" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G214" s="7" t="inlineStr"/>
     </row>
     <row r="215">
@@ -4524,7 +4949,9 @@
       </c>
       <c r="D215" s="7" t="inlineStr"/>
       <c r="E215" s="7" t="inlineStr"/>
-      <c r="F215" s="7" t="inlineStr"/>
+      <c r="F215" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G215" s="7" t="inlineStr"/>
     </row>
     <row r="216">
@@ -4543,7 +4970,9 @@
       </c>
       <c r="D216" s="7" t="inlineStr"/>
       <c r="E216" s="7" t="inlineStr"/>
-      <c r="F216" s="7" t="inlineStr"/>
+      <c r="F216" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G216" s="7" t="inlineStr"/>
     </row>
     <row r="217">
@@ -4562,7 +4991,9 @@
       </c>
       <c r="D217" s="7" t="inlineStr"/>
       <c r="E217" s="7" t="inlineStr"/>
-      <c r="F217" s="7" t="inlineStr"/>
+      <c r="F217" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G217" s="7" t="inlineStr"/>
     </row>
     <row r="218">
@@ -4581,7 +5012,9 @@
       </c>
       <c r="D218" s="7" t="inlineStr"/>
       <c r="E218" s="7" t="inlineStr"/>
-      <c r="F218" s="7" t="inlineStr"/>
+      <c r="F218" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G218" s="7" t="inlineStr"/>
     </row>
     <row r="219">
@@ -4600,7 +5033,9 @@
       </c>
       <c r="D219" s="7" t="inlineStr"/>
       <c r="E219" s="7" t="inlineStr"/>
-      <c r="F219" s="7" t="inlineStr"/>
+      <c r="F219" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G219" s="7" t="inlineStr"/>
     </row>
     <row r="220">
@@ -4615,7 +5050,9 @@
       <c r="C220" s="5" t="inlineStr"/>
       <c r="D220" s="7" t="inlineStr"/>
       <c r="E220" s="7" t="inlineStr"/>
-      <c r="F220" s="7" t="inlineStr"/>
+      <c r="F220" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G220" s="7" t="inlineStr"/>
     </row>
     <row r="221">
@@ -4630,7 +5067,9 @@
       <c r="C221" s="5" t="inlineStr"/>
       <c r="D221" s="7" t="inlineStr"/>
       <c r="E221" s="7" t="inlineStr"/>
-      <c r="F221" s="7" t="inlineStr"/>
+      <c r="F221" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G221" s="7" t="inlineStr"/>
     </row>
     <row r="222">
@@ -4645,7 +5084,9 @@
       <c r="C222" s="5" t="inlineStr"/>
       <c r="D222" s="7" t="inlineStr"/>
       <c r="E222" s="7" t="inlineStr"/>
-      <c r="F222" s="7" t="inlineStr"/>
+      <c r="F222" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G222" s="7" t="inlineStr"/>
     </row>
     <row r="223">
@@ -4664,7 +5105,9 @@
       </c>
       <c r="D223" s="7" t="inlineStr"/>
       <c r="E223" s="7" t="inlineStr"/>
-      <c r="F223" s="7" t="inlineStr"/>
+      <c r="F223" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G223" s="7" t="inlineStr"/>
     </row>
     <row r="224">
@@ -4683,7 +5126,9 @@
       </c>
       <c r="D224" s="7" t="inlineStr"/>
       <c r="E224" s="7" t="inlineStr"/>
-      <c r="F224" s="7" t="inlineStr"/>
+      <c r="F224" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G224" s="7" t="inlineStr"/>
     </row>
     <row r="225">
@@ -4702,7 +5147,9 @@
       </c>
       <c r="D225" s="7" t="inlineStr"/>
       <c r="E225" s="7" t="inlineStr"/>
-      <c r="F225" s="7" t="inlineStr"/>
+      <c r="F225" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G225" s="7" t="inlineStr"/>
     </row>
     <row r="226">
@@ -4721,7 +5168,9 @@
       </c>
       <c r="D226" s="7" t="inlineStr"/>
       <c r="E226" s="7" t="inlineStr"/>
-      <c r="F226" s="7" t="inlineStr"/>
+      <c r="F226" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G226" s="7" t="inlineStr"/>
     </row>
     <row r="227">
@@ -4740,7 +5189,9 @@
       </c>
       <c r="D227" s="7" t="inlineStr"/>
       <c r="E227" s="7" t="inlineStr"/>
-      <c r="F227" s="7" t="inlineStr"/>
+      <c r="F227" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G227" s="7" t="inlineStr"/>
     </row>
     <row r="228">
@@ -4755,7 +5206,9 @@
       <c r="C228" s="5" t="inlineStr"/>
       <c r="D228" s="7" t="inlineStr"/>
       <c r="E228" s="7" t="inlineStr"/>
-      <c r="F228" s="7" t="inlineStr"/>
+      <c r="F228" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G228" s="7" t="inlineStr"/>
     </row>
     <row r="229">
@@ -4774,7 +5227,9 @@
       </c>
       <c r="D229" s="7" t="inlineStr"/>
       <c r="E229" s="7" t="inlineStr"/>
-      <c r="F229" s="7" t="inlineStr"/>
+      <c r="F229" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G229" s="7" t="inlineStr"/>
     </row>
     <row r="230">
@@ -4789,7 +5244,9 @@
       <c r="C230" s="5" t="inlineStr"/>
       <c r="D230" s="7" t="inlineStr"/>
       <c r="E230" s="7" t="inlineStr"/>
-      <c r="F230" s="7" t="inlineStr"/>
+      <c r="F230" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G230" s="7" t="inlineStr"/>
     </row>
     <row r="231">
@@ -4808,7 +5265,9 @@
       </c>
       <c r="D231" s="7" t="inlineStr"/>
       <c r="E231" s="7" t="inlineStr"/>
-      <c r="F231" s="7" t="inlineStr"/>
+      <c r="F231" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G231" s="7" t="inlineStr"/>
     </row>
     <row r="232">
@@ -4827,7 +5286,9 @@
       </c>
       <c r="D232" s="7" t="inlineStr"/>
       <c r="E232" s="7" t="inlineStr"/>
-      <c r="F232" s="7" t="inlineStr"/>
+      <c r="F232" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G232" s="7" t="inlineStr"/>
     </row>
     <row r="233">
@@ -4846,7 +5307,9 @@
       </c>
       <c r="D233" s="7" t="inlineStr"/>
       <c r="E233" s="7" t="inlineStr"/>
-      <c r="F233" s="7" t="inlineStr"/>
+      <c r="F233" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G233" s="7" t="inlineStr"/>
     </row>
     <row r="234">
@@ -4865,7 +5328,9 @@
       </c>
       <c r="D234" s="7" t="inlineStr"/>
       <c r="E234" s="7" t="inlineStr"/>
-      <c r="F234" s="7" t="inlineStr"/>
+      <c r="F234" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G234" s="7" t="inlineStr"/>
     </row>
     <row r="235">
@@ -4884,7 +5349,9 @@
       </c>
       <c r="D235" s="7" t="inlineStr"/>
       <c r="E235" s="7" t="inlineStr"/>
-      <c r="F235" s="7" t="inlineStr"/>
+      <c r="F235" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G235" s="7" t="inlineStr"/>
     </row>
     <row r="236">
@@ -4903,7 +5370,9 @@
       </c>
       <c r="D236" s="7" t="inlineStr"/>
       <c r="E236" s="7" t="inlineStr"/>
-      <c r="F236" s="7" t="inlineStr"/>
+      <c r="F236" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G236" s="7" t="inlineStr"/>
     </row>
     <row r="237">
@@ -4922,7 +5391,9 @@
       </c>
       <c r="D237" s="7" t="inlineStr"/>
       <c r="E237" s="7" t="inlineStr"/>
-      <c r="F237" s="7" t="inlineStr"/>
+      <c r="F237" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G237" s="7" t="inlineStr"/>
     </row>
     <row r="238">
@@ -4941,7 +5412,9 @@
       </c>
       <c r="D238" s="7" t="inlineStr"/>
       <c r="E238" s="7" t="inlineStr"/>
-      <c r="F238" s="7" t="inlineStr"/>
+      <c r="F238" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G238" s="7" t="inlineStr"/>
     </row>
     <row r="239">
@@ -4960,7 +5433,9 @@
       </c>
       <c r="D239" s="7" t="inlineStr"/>
       <c r="E239" s="7" t="inlineStr"/>
-      <c r="F239" s="7" t="inlineStr"/>
+      <c r="F239" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G239" s="7" t="inlineStr"/>
     </row>
     <row r="240">
@@ -4975,7 +5450,9 @@
       <c r="C240" s="5" t="inlineStr"/>
       <c r="D240" s="7" t="inlineStr"/>
       <c r="E240" s="7" t="inlineStr"/>
-      <c r="F240" s="7" t="inlineStr"/>
+      <c r="F240" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G240" s="7" t="inlineStr"/>
     </row>
     <row r="241">
@@ -4994,7 +5471,9 @@
       </c>
       <c r="D241" s="7" t="inlineStr"/>
       <c r="E241" s="7" t="inlineStr"/>
-      <c r="F241" s="7" t="inlineStr"/>
+      <c r="F241" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G241" s="7" t="inlineStr"/>
     </row>
     <row r="242">
@@ -5013,7 +5492,9 @@
       </c>
       <c r="D242" s="7" t="inlineStr"/>
       <c r="E242" s="7" t="inlineStr"/>
-      <c r="F242" s="7" t="inlineStr"/>
+      <c r="F242" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G242" s="7" t="inlineStr"/>
     </row>
     <row r="243">
@@ -5032,7 +5513,9 @@
       </c>
       <c r="D243" s="7" t="inlineStr"/>
       <c r="E243" s="7" t="inlineStr"/>
-      <c r="F243" s="7" t="inlineStr"/>
+      <c r="F243" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G243" s="7" t="inlineStr"/>
     </row>
     <row r="244">
@@ -5051,7 +5534,9 @@
       </c>
       <c r="D244" s="7" t="inlineStr"/>
       <c r="E244" s="7" t="inlineStr"/>
-      <c r="F244" s="7" t="inlineStr"/>
+      <c r="F244" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G244" s="7" t="inlineStr"/>
     </row>
     <row r="245">
@@ -5070,7 +5555,9 @@
       </c>
       <c r="D245" s="7" t="inlineStr"/>
       <c r="E245" s="7" t="inlineStr"/>
-      <c r="F245" s="7" t="inlineStr"/>
+      <c r="F245" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G245" s="7" t="inlineStr"/>
     </row>
     <row r="246">
@@ -5089,7 +5576,9 @@
       </c>
       <c r="D246" s="7" t="inlineStr"/>
       <c r="E246" s="7" t="inlineStr"/>
-      <c r="F246" s="7" t="inlineStr"/>
+      <c r="F246" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G246" s="7" t="inlineStr"/>
     </row>
     <row r="247">
@@ -5108,7 +5597,9 @@
       </c>
       <c r="D247" s="7" t="inlineStr"/>
       <c r="E247" s="7" t="inlineStr"/>
-      <c r="F247" s="7" t="inlineStr"/>
+      <c r="F247" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G247" s="7" t="inlineStr"/>
     </row>
     <row r="248">
@@ -5127,7 +5618,9 @@
       </c>
       <c r="D248" s="7" t="inlineStr"/>
       <c r="E248" s="7" t="inlineStr"/>
-      <c r="F248" s="7" t="inlineStr"/>
+      <c r="F248" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G248" s="7" t="inlineStr"/>
     </row>
     <row r="249">
@@ -5146,7 +5639,9 @@
       </c>
       <c r="D249" s="7" t="inlineStr"/>
       <c r="E249" s="7" t="inlineStr"/>
-      <c r="F249" s="7" t="inlineStr"/>
+      <c r="F249" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G249" s="7" t="inlineStr"/>
     </row>
     <row r="250">
@@ -5161,7 +5656,9 @@
       <c r="C250" s="5" t="inlineStr"/>
       <c r="D250" s="7" t="inlineStr"/>
       <c r="E250" s="7" t="inlineStr"/>
-      <c r="F250" s="7" t="inlineStr"/>
+      <c r="F250" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G250" s="7" t="inlineStr"/>
     </row>
     <row r="251">
@@ -5180,7 +5677,9 @@
       </c>
       <c r="D251" s="7" t="inlineStr"/>
       <c r="E251" s="7" t="inlineStr"/>
-      <c r="F251" s="7" t="inlineStr"/>
+      <c r="F251" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G251" s="7" t="inlineStr"/>
     </row>
     <row r="252">
@@ -5199,7 +5698,9 @@
       </c>
       <c r="D252" s="7" t="inlineStr"/>
       <c r="E252" s="7" t="inlineStr"/>
-      <c r="F252" s="7" t="inlineStr"/>
+      <c r="F252" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G252" s="7" t="inlineStr"/>
     </row>
     <row r="253">
@@ -5218,7 +5719,9 @@
       </c>
       <c r="D253" s="7" t="inlineStr"/>
       <c r="E253" s="7" t="inlineStr"/>
-      <c r="F253" s="7" t="inlineStr"/>
+      <c r="F253" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G253" s="7" t="inlineStr"/>
     </row>
     <row r="254">
@@ -5237,7 +5740,9 @@
       </c>
       <c r="D254" s="7" t="inlineStr"/>
       <c r="E254" s="7" t="inlineStr"/>
-      <c r="F254" s="7" t="inlineStr"/>
+      <c r="F254" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G254" s="7" t="inlineStr"/>
     </row>
     <row r="255">
@@ -5256,7 +5761,9 @@
       </c>
       <c r="D255" s="7" t="inlineStr"/>
       <c r="E255" s="7" t="inlineStr"/>
-      <c r="F255" s="7" t="inlineStr"/>
+      <c r="F255" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G255" s="7" t="inlineStr"/>
     </row>
     <row r="256">
@@ -5275,7 +5782,9 @@
       </c>
       <c r="D256" s="7" t="inlineStr"/>
       <c r="E256" s="7" t="inlineStr"/>
-      <c r="F256" s="7" t="inlineStr"/>
+      <c r="F256" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G256" s="7" t="inlineStr"/>
     </row>
     <row r="257">
@@ -5294,7 +5803,9 @@
       </c>
       <c r="D257" s="7" t="inlineStr"/>
       <c r="E257" s="7" t="inlineStr"/>
-      <c r="F257" s="7" t="inlineStr"/>
+      <c r="F257" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G257" s="7" t="inlineStr"/>
     </row>
     <row r="258">
@@ -5313,7 +5824,9 @@
       </c>
       <c r="D258" s="7" t="inlineStr"/>
       <c r="E258" s="7" t="inlineStr"/>
-      <c r="F258" s="7" t="inlineStr"/>
+      <c r="F258" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G258" s="7" t="inlineStr"/>
     </row>
     <row r="259">
@@ -5332,7 +5845,9 @@
       </c>
       <c r="D259" s="7" t="inlineStr"/>
       <c r="E259" s="7" t="inlineStr"/>
-      <c r="F259" s="7" t="inlineStr"/>
+      <c r="F259" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G259" s="7" t="inlineStr"/>
     </row>
     <row r="260">
@@ -5351,7 +5866,9 @@
       </c>
       <c r="D260" s="7" t="inlineStr"/>
       <c r="E260" s="7" t="inlineStr"/>
-      <c r="F260" s="7" t="inlineStr"/>
+      <c r="F260" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G260" s="7" t="inlineStr"/>
     </row>
     <row r="261">
@@ -5370,7 +5887,9 @@
       </c>
       <c r="D261" s="7" t="inlineStr"/>
       <c r="E261" s="7" t="inlineStr"/>
-      <c r="F261" s="7" t="inlineStr"/>
+      <c r="F261" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G261" s="7" t="inlineStr"/>
     </row>
     <row r="262">
@@ -5389,7 +5908,9 @@
       </c>
       <c r="D262" s="7" t="inlineStr"/>
       <c r="E262" s="7" t="inlineStr"/>
-      <c r="F262" s="7" t="inlineStr"/>
+      <c r="F262" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G262" s="7" t="inlineStr"/>
     </row>
     <row r="263">
@@ -5408,7 +5929,9 @@
       </c>
       <c r="D263" s="7" t="inlineStr"/>
       <c r="E263" s="7" t="inlineStr"/>
-      <c r="F263" s="7" t="inlineStr"/>
+      <c r="F263" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G263" s="7" t="inlineStr"/>
     </row>
     <row r="264">
@@ -5427,7 +5950,9 @@
       </c>
       <c r="D264" s="7" t="inlineStr"/>
       <c r="E264" s="7" t="inlineStr"/>
-      <c r="F264" s="7" t="inlineStr"/>
+      <c r="F264" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G264" s="7" t="inlineStr"/>
     </row>
     <row r="265">
@@ -5446,7 +5971,9 @@
       </c>
       <c r="D265" s="7" t="inlineStr"/>
       <c r="E265" s="7" t="inlineStr"/>
-      <c r="F265" s="7" t="inlineStr"/>
+      <c r="F265" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G265" s="7" t="inlineStr"/>
     </row>
     <row r="266">
@@ -5465,7 +5992,9 @@
       </c>
       <c r="D266" s="7" t="inlineStr"/>
       <c r="E266" s="7" t="inlineStr"/>
-      <c r="F266" s="7" t="inlineStr"/>
+      <c r="F266" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G266" s="7" t="inlineStr"/>
     </row>
     <row r="267">
@@ -5484,7 +6013,9 @@
       </c>
       <c r="D267" s="7" t="inlineStr"/>
       <c r="E267" s="7" t="inlineStr"/>
-      <c r="F267" s="7" t="inlineStr"/>
+      <c r="F267" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G267" s="7" t="inlineStr"/>
     </row>
     <row r="268">
@@ -5503,7 +6034,9 @@
       </c>
       <c r="D268" s="7" t="inlineStr"/>
       <c r="E268" s="7" t="inlineStr"/>
-      <c r="F268" s="7" t="inlineStr"/>
+      <c r="F268" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G268" s="7" t="inlineStr"/>
     </row>
     <row r="269">
@@ -5522,7 +6055,9 @@
       </c>
       <c r="D269" s="7" t="inlineStr"/>
       <c r="E269" s="7" t="inlineStr"/>
-      <c r="F269" s="7" t="inlineStr"/>
+      <c r="F269" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G269" s="7" t="inlineStr"/>
     </row>
     <row r="270">
@@ -5541,7 +6076,9 @@
       </c>
       <c r="D270" s="7" t="inlineStr"/>
       <c r="E270" s="7" t="inlineStr"/>
-      <c r="F270" s="7" t="inlineStr"/>
+      <c r="F270" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G270" s="7" t="inlineStr"/>
     </row>
     <row r="271">
@@ -5560,7 +6097,9 @@
       </c>
       <c r="D271" s="7" t="inlineStr"/>
       <c r="E271" s="7" t="inlineStr"/>
-      <c r="F271" s="7" t="inlineStr"/>
+      <c r="F271" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G271" s="7" t="inlineStr"/>
     </row>
     <row r="272">
@@ -5579,7 +6118,9 @@
       </c>
       <c r="D272" s="7" t="inlineStr"/>
       <c r="E272" s="7" t="inlineStr"/>
-      <c r="F272" s="7" t="inlineStr"/>
+      <c r="F272" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G272" s="7" t="inlineStr"/>
     </row>
     <row r="273">
@@ -5598,7 +6139,9 @@
       </c>
       <c r="D273" s="7" t="inlineStr"/>
       <c r="E273" s="7" t="inlineStr"/>
-      <c r="F273" s="7" t="inlineStr"/>
+      <c r="F273" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G273" s="7" t="inlineStr"/>
     </row>
     <row r="274">
@@ -5617,7 +6160,9 @@
       </c>
       <c r="D274" s="7" t="inlineStr"/>
       <c r="E274" s="7" t="inlineStr"/>
-      <c r="F274" s="7" t="inlineStr"/>
+      <c r="F274" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G274" s="7" t="inlineStr"/>
     </row>
     <row r="275">
@@ -5636,7 +6181,9 @@
       </c>
       <c r="D275" s="7" t="inlineStr"/>
       <c r="E275" s="7" t="inlineStr"/>
-      <c r="F275" s="7" t="inlineStr"/>
+      <c r="F275" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G275" s="7" t="inlineStr"/>
     </row>
     <row r="276">
@@ -5655,7 +6202,9 @@
       </c>
       <c r="D276" s="7" t="inlineStr"/>
       <c r="E276" s="7" t="inlineStr"/>
-      <c r="F276" s="7" t="inlineStr"/>
+      <c r="F276" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G276" s="7" t="inlineStr"/>
     </row>
     <row r="277">
@@ -5674,7 +6223,9 @@
       </c>
       <c r="D277" s="7" t="inlineStr"/>
       <c r="E277" s="7" t="inlineStr"/>
-      <c r="F277" s="7" t="inlineStr"/>
+      <c r="F277" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G277" s="7" t="inlineStr"/>
     </row>
     <row r="278">
@@ -5693,7 +6244,9 @@
       </c>
       <c r="D278" s="7" t="inlineStr"/>
       <c r="E278" s="7" t="inlineStr"/>
-      <c r="F278" s="7" t="inlineStr"/>
+      <c r="F278" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G278" s="7" t="inlineStr"/>
     </row>
     <row r="279">
@@ -5712,7 +6265,9 @@
       </c>
       <c r="D279" s="7" t="inlineStr"/>
       <c r="E279" s="7" t="inlineStr"/>
-      <c r="F279" s="7" t="inlineStr"/>
+      <c r="F279" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G279" s="7" t="inlineStr"/>
     </row>
     <row r="280">
@@ -5731,7 +6286,9 @@
       </c>
       <c r="D280" s="7" t="inlineStr"/>
       <c r="E280" s="7" t="inlineStr"/>
-      <c r="F280" s="7" t="inlineStr"/>
+      <c r="F280" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G280" s="7" t="inlineStr"/>
     </row>
     <row r="281">
@@ -5750,7 +6307,9 @@
       </c>
       <c r="D281" s="7" t="inlineStr"/>
       <c r="E281" s="7" t="inlineStr"/>
-      <c r="F281" s="7" t="inlineStr"/>
+      <c r="F281" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G281" s="7" t="inlineStr"/>
     </row>
     <row r="282">
@@ -5769,7 +6328,9 @@
       </c>
       <c r="D282" s="7" t="inlineStr"/>
       <c r="E282" s="7" t="inlineStr"/>
-      <c r="F282" s="7" t="inlineStr"/>
+      <c r="F282" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G282" s="7" t="inlineStr"/>
     </row>
     <row r="283">
@@ -5788,7 +6349,9 @@
       </c>
       <c r="D283" s="7" t="inlineStr"/>
       <c r="E283" s="7" t="inlineStr"/>
-      <c r="F283" s="7" t="inlineStr"/>
+      <c r="F283" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G283" s="7" t="inlineStr"/>
     </row>
     <row r="284">
@@ -5807,7 +6370,9 @@
       </c>
       <c r="D284" s="7" t="inlineStr"/>
       <c r="E284" s="7" t="inlineStr"/>
-      <c r="F284" s="7" t="inlineStr"/>
+      <c r="F284" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G284" s="7" t="inlineStr"/>
     </row>
     <row r="285">
@@ -5826,7 +6391,9 @@
       </c>
       <c r="D285" s="7" t="inlineStr"/>
       <c r="E285" s="7" t="inlineStr"/>
-      <c r="F285" s="7" t="inlineStr"/>
+      <c r="F285" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G285" s="7" t="inlineStr"/>
     </row>
     <row r="286">
@@ -5845,7 +6412,9 @@
       </c>
       <c r="D286" s="7" t="inlineStr"/>
       <c r="E286" s="7" t="inlineStr"/>
-      <c r="F286" s="7" t="inlineStr"/>
+      <c r="F286" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G286" s="7" t="inlineStr"/>
     </row>
     <row r="287">
@@ -5864,7 +6433,9 @@
       </c>
       <c r="D287" s="7" t="inlineStr"/>
       <c r="E287" s="7" t="inlineStr"/>
-      <c r="F287" s="7" t="inlineStr"/>
+      <c r="F287" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G287" s="7" t="inlineStr"/>
     </row>
     <row r="288">
@@ -5883,7 +6454,9 @@
       </c>
       <c r="D288" s="7" t="inlineStr"/>
       <c r="E288" s="7" t="inlineStr"/>
-      <c r="F288" s="7" t="inlineStr"/>
+      <c r="F288" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G288" s="7" t="inlineStr"/>
     </row>
     <row r="289">
@@ -5902,7 +6475,9 @@
       </c>
       <c r="D289" s="7" t="inlineStr"/>
       <c r="E289" s="7" t="inlineStr"/>
-      <c r="F289" s="7" t="inlineStr"/>
+      <c r="F289" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G289" s="7" t="inlineStr"/>
     </row>
     <row r="290">
@@ -5921,7 +6496,9 @@
       </c>
       <c r="D290" s="7" t="inlineStr"/>
       <c r="E290" s="7" t="inlineStr"/>
-      <c r="F290" s="7" t="inlineStr"/>
+      <c r="F290" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G290" s="7" t="inlineStr"/>
     </row>
     <row r="291">
@@ -5940,7 +6517,9 @@
       </c>
       <c r="D291" s="7" t="inlineStr"/>
       <c r="E291" s="7" t="inlineStr"/>
-      <c r="F291" s="7" t="inlineStr"/>
+      <c r="F291" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G291" s="7" t="inlineStr"/>
     </row>
     <row r="292">
@@ -5955,7 +6534,9 @@
       <c r="C292" s="5" t="inlineStr"/>
       <c r="D292" s="7" t="inlineStr"/>
       <c r="E292" s="7" t="inlineStr"/>
-      <c r="F292" s="7" t="inlineStr"/>
+      <c r="F292" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G292" s="7" t="inlineStr"/>
     </row>
     <row r="293">
@@ -5974,7 +6555,9 @@
       </c>
       <c r="D293" s="7" t="inlineStr"/>
       <c r="E293" s="7" t="inlineStr"/>
-      <c r="F293" s="7" t="inlineStr"/>
+      <c r="F293" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G293" s="7" t="inlineStr"/>
     </row>
     <row r="294">
@@ -5993,7 +6576,9 @@
       </c>
       <c r="D294" s="7" t="inlineStr"/>
       <c r="E294" s="7" t="inlineStr"/>
-      <c r="F294" s="7" t="inlineStr"/>
+      <c r="F294" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G294" s="7" t="inlineStr"/>
     </row>
     <row r="295">
@@ -6012,7 +6597,9 @@
       </c>
       <c r="D295" s="7" t="inlineStr"/>
       <c r="E295" s="7" t="inlineStr"/>
-      <c r="F295" s="7" t="inlineStr"/>
+      <c r="F295" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G295" s="7" t="inlineStr"/>
     </row>
     <row r="296">
@@ -6031,7 +6618,9 @@
       </c>
       <c r="D296" s="7" t="inlineStr"/>
       <c r="E296" s="7" t="inlineStr"/>
-      <c r="F296" s="7" t="inlineStr"/>
+      <c r="F296" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G296" s="7" t="inlineStr"/>
     </row>
     <row r="297">
@@ -6050,7 +6639,9 @@
       </c>
       <c r="D297" s="7" t="inlineStr"/>
       <c r="E297" s="7" t="inlineStr"/>
-      <c r="F297" s="7" t="inlineStr"/>
+      <c r="F297" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G297" s="7" t="inlineStr"/>
     </row>
     <row r="298">
@@ -6069,7 +6660,9 @@
       </c>
       <c r="D298" s="7" t="inlineStr"/>
       <c r="E298" s="7" t="inlineStr"/>
-      <c r="F298" s="7" t="inlineStr"/>
+      <c r="F298" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G298" s="7" t="inlineStr"/>
     </row>
     <row r="299">
@@ -6088,7 +6681,9 @@
       </c>
       <c r="D299" s="7" t="inlineStr"/>
       <c r="E299" s="7" t="inlineStr"/>
-      <c r="F299" s="7" t="inlineStr"/>
+      <c r="F299" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G299" s="7" t="inlineStr"/>
     </row>
     <row r="300">
@@ -6107,7 +6702,9 @@
       </c>
       <c r="D300" s="7" t="inlineStr"/>
       <c r="E300" s="7" t="inlineStr"/>
-      <c r="F300" s="7" t="inlineStr"/>
+      <c r="F300" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G300" s="7" t="inlineStr"/>
     </row>
     <row r="301">
@@ -6126,7 +6723,9 @@
       </c>
       <c r="D301" s="7" t="inlineStr"/>
       <c r="E301" s="7" t="inlineStr"/>
-      <c r="F301" s="7" t="inlineStr"/>
+      <c r="F301" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G301" s="7" t="inlineStr"/>
     </row>
     <row r="302">
@@ -6145,7 +6744,9 @@
       </c>
       <c r="D302" s="7" t="inlineStr"/>
       <c r="E302" s="7" t="inlineStr"/>
-      <c r="F302" s="7" t="inlineStr"/>
+      <c r="F302" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G302" s="7" t="inlineStr"/>
     </row>
     <row r="303">
@@ -6164,7 +6765,9 @@
       </c>
       <c r="D303" s="7" t="inlineStr"/>
       <c r="E303" s="7" t="inlineStr"/>
-      <c r="F303" s="7" t="inlineStr"/>
+      <c r="F303" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G303" s="7" t="inlineStr"/>
     </row>
     <row r="304">
@@ -6183,7 +6786,9 @@
       </c>
       <c r="D304" s="7" t="inlineStr"/>
       <c r="E304" s="7" t="inlineStr"/>
-      <c r="F304" s="7" t="inlineStr"/>
+      <c r="F304" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G304" s="7" t="inlineStr"/>
     </row>
     <row r="305">
@@ -6198,7 +6803,9 @@
       <c r="C305" s="5" t="inlineStr"/>
       <c r="D305" s="7" t="inlineStr"/>
       <c r="E305" s="7" t="inlineStr"/>
-      <c r="F305" s="7" t="inlineStr"/>
+      <c r="F305" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G305" s="7" t="inlineStr"/>
     </row>
     <row r="306">
@@ -6217,7 +6824,9 @@
       </c>
       <c r="D306" s="7" t="inlineStr"/>
       <c r="E306" s="7" t="inlineStr"/>
-      <c r="F306" s="7" t="inlineStr"/>
+      <c r="F306" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G306" s="7" t="inlineStr"/>
     </row>
     <row r="307">
@@ -6236,7 +6845,9 @@
       </c>
       <c r="D307" s="7" t="inlineStr"/>
       <c r="E307" s="7" t="inlineStr"/>
-      <c r="F307" s="7" t="inlineStr"/>
+      <c r="F307" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G307" s="7" t="inlineStr"/>
     </row>
     <row r="308">
@@ -6255,7 +6866,9 @@
       </c>
       <c r="D308" s="7" t="inlineStr"/>
       <c r="E308" s="7" t="inlineStr"/>
-      <c r="F308" s="7" t="inlineStr"/>
+      <c r="F308" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G308" s="7" t="inlineStr"/>
     </row>
     <row r="309">
@@ -6274,7 +6887,9 @@
       </c>
       <c r="D309" s="7" t="inlineStr"/>
       <c r="E309" s="7" t="inlineStr"/>
-      <c r="F309" s="7" t="inlineStr"/>
+      <c r="F309" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G309" s="7" t="inlineStr"/>
     </row>
     <row r="310">
@@ -6293,7 +6908,9 @@
       </c>
       <c r="D310" s="7" t="inlineStr"/>
       <c r="E310" s="7" t="inlineStr"/>
-      <c r="F310" s="7" t="inlineStr"/>
+      <c r="F310" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G310" s="7" t="inlineStr"/>
     </row>
     <row r="311">
@@ -6312,7 +6929,9 @@
       </c>
       <c r="D311" s="7" t="inlineStr"/>
       <c r="E311" s="7" t="inlineStr"/>
-      <c r="F311" s="7" t="inlineStr"/>
+      <c r="F311" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G311" s="7" t="inlineStr"/>
     </row>
     <row r="312">
@@ -6331,7 +6950,9 @@
       </c>
       <c r="D312" s="7" t="inlineStr"/>
       <c r="E312" s="7" t="inlineStr"/>
-      <c r="F312" s="7" t="inlineStr"/>
+      <c r="F312" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G312" s="7" t="inlineStr"/>
     </row>
     <row r="313">
@@ -6350,7 +6971,9 @@
       </c>
       <c r="D313" s="7" t="inlineStr"/>
       <c r="E313" s="7" t="inlineStr"/>
-      <c r="F313" s="7" t="inlineStr"/>
+      <c r="F313" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G313" s="7" t="inlineStr"/>
     </row>
     <row r="314">
@@ -6369,7 +6992,9 @@
       </c>
       <c r="D314" s="7" t="inlineStr"/>
       <c r="E314" s="7" t="inlineStr"/>
-      <c r="F314" s="7" t="inlineStr"/>
+      <c r="F314" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G314" s="7" t="inlineStr"/>
     </row>
     <row r="315">
@@ -6388,7 +7013,9 @@
       </c>
       <c r="D315" s="7" t="inlineStr"/>
       <c r="E315" s="7" t="inlineStr"/>
-      <c r="F315" s="7" t="inlineStr"/>
+      <c r="F315" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G315" s="7" t="inlineStr"/>
     </row>
     <row r="316">
@@ -6407,7 +7034,9 @@
       </c>
       <c r="D316" s="7" t="inlineStr"/>
       <c r="E316" s="7" t="inlineStr"/>
-      <c r="F316" s="7" t="inlineStr"/>
+      <c r="F316" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G316" s="7" t="inlineStr"/>
     </row>
     <row r="317">
@@ -6426,7 +7055,9 @@
       </c>
       <c r="D317" s="7" t="inlineStr"/>
       <c r="E317" s="7" t="inlineStr"/>
-      <c r="F317" s="7" t="inlineStr"/>
+      <c r="F317" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G317" s="7" t="inlineStr"/>
     </row>
     <row r="318">
@@ -6445,7 +7076,9 @@
       </c>
       <c r="D318" s="7" t="inlineStr"/>
       <c r="E318" s="7" t="inlineStr"/>
-      <c r="F318" s="7" t="inlineStr"/>
+      <c r="F318" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G318" s="7" t="inlineStr"/>
     </row>
     <row r="319">
@@ -6464,7 +7097,9 @@
       </c>
       <c r="D319" s="7" t="inlineStr"/>
       <c r="E319" s="7" t="inlineStr"/>
-      <c r="F319" s="7" t="inlineStr"/>
+      <c r="F319" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G319" s="7" t="inlineStr"/>
     </row>
     <row r="320">
@@ -6483,7 +7118,9 @@
       </c>
       <c r="D320" s="7" t="inlineStr"/>
       <c r="E320" s="7" t="inlineStr"/>
-      <c r="F320" s="7" t="inlineStr"/>
+      <c r="F320" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G320" s="7" t="inlineStr"/>
     </row>
     <row r="321">
@@ -6502,7 +7139,9 @@
       </c>
       <c r="D321" s="7" t="inlineStr"/>
       <c r="E321" s="7" t="inlineStr"/>
-      <c r="F321" s="7" t="inlineStr"/>
+      <c r="F321" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G321" s="7" t="inlineStr"/>
     </row>
     <row r="322">
@@ -6517,7 +7156,9 @@
       <c r="C322" s="5" t="inlineStr"/>
       <c r="D322" s="7" t="inlineStr"/>
       <c r="E322" s="7" t="inlineStr"/>
-      <c r="F322" s="7" t="inlineStr"/>
+      <c r="F322" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G322" s="7" t="inlineStr"/>
     </row>
     <row r="323">
@@ -6536,7 +7177,9 @@
       </c>
       <c r="D323" s="7" t="inlineStr"/>
       <c r="E323" s="7" t="inlineStr"/>
-      <c r="F323" s="7" t="inlineStr"/>
+      <c r="F323" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G323" s="7" t="inlineStr"/>
     </row>
     <row r="324">
@@ -6555,7 +7198,9 @@
       </c>
       <c r="D324" s="7" t="inlineStr"/>
       <c r="E324" s="7" t="inlineStr"/>
-      <c r="F324" s="7" t="inlineStr"/>
+      <c r="F324" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G324" s="7" t="inlineStr"/>
     </row>
     <row r="325">
@@ -6574,7 +7219,9 @@
       </c>
       <c r="D325" s="7" t="inlineStr"/>
       <c r="E325" s="7" t="inlineStr"/>
-      <c r="F325" s="7" t="inlineStr"/>
+      <c r="F325" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G325" s="7" t="inlineStr"/>
     </row>
     <row r="326">
@@ -6593,7 +7240,9 @@
       </c>
       <c r="D326" s="7" t="inlineStr"/>
       <c r="E326" s="7" t="inlineStr"/>
-      <c r="F326" s="7" t="inlineStr"/>
+      <c r="F326" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G326" s="7" t="inlineStr"/>
     </row>
     <row r="327">
@@ -6612,7 +7261,9 @@
       </c>
       <c r="D327" s="7" t="inlineStr"/>
       <c r="E327" s="7" t="inlineStr"/>
-      <c r="F327" s="7" t="inlineStr"/>
+      <c r="F327" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G327" s="7" t="inlineStr"/>
     </row>
     <row r="328">
@@ -6631,7 +7282,9 @@
       </c>
       <c r="D328" s="7" t="inlineStr"/>
       <c r="E328" s="7" t="inlineStr"/>
-      <c r="F328" s="7" t="inlineStr"/>
+      <c r="F328" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G328" s="7" t="inlineStr"/>
     </row>
     <row r="329">
@@ -6650,7 +7303,9 @@
       </c>
       <c r="D329" s="7" t="inlineStr"/>
       <c r="E329" s="7" t="inlineStr"/>
-      <c r="F329" s="7" t="inlineStr"/>
+      <c r="F329" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G329" s="7" t="inlineStr"/>
     </row>
     <row r="330">
@@ -6669,7 +7324,9 @@
       </c>
       <c r="D330" s="7" t="inlineStr"/>
       <c r="E330" s="7" t="inlineStr"/>
-      <c r="F330" s="7" t="inlineStr"/>
+      <c r="F330" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G330" s="7" t="inlineStr"/>
     </row>
     <row r="331">
@@ -6688,7 +7345,9 @@
       </c>
       <c r="D331" s="7" t="inlineStr"/>
       <c r="E331" s="7" t="inlineStr"/>
-      <c r="F331" s="7" t="inlineStr"/>
+      <c r="F331" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G331" s="7" t="inlineStr"/>
     </row>
     <row r="332">
@@ -6707,7 +7366,9 @@
       </c>
       <c r="D332" s="7" t="inlineStr"/>
       <c r="E332" s="7" t="inlineStr"/>
-      <c r="F332" s="7" t="inlineStr"/>
+      <c r="F332" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G332" s="7" t="inlineStr"/>
     </row>
     <row r="333">
@@ -6726,7 +7387,9 @@
       </c>
       <c r="D333" s="7" t="inlineStr"/>
       <c r="E333" s="7" t="inlineStr"/>
-      <c r="F333" s="7" t="inlineStr"/>
+      <c r="F333" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G333" s="7" t="inlineStr"/>
     </row>
     <row r="334">
@@ -6745,7 +7408,9 @@
       </c>
       <c r="D334" s="7" t="inlineStr"/>
       <c r="E334" s="7" t="inlineStr"/>
-      <c r="F334" s="7" t="inlineStr"/>
+      <c r="F334" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G334" s="7" t="inlineStr"/>
     </row>
     <row r="335">
@@ -6764,7 +7429,9 @@
       </c>
       <c r="D335" s="7" t="inlineStr"/>
       <c r="E335" s="7" t="inlineStr"/>
-      <c r="F335" s="7" t="inlineStr"/>
+      <c r="F335" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G335" s="7" t="inlineStr"/>
     </row>
     <row r="336">
@@ -6783,7 +7450,9 @@
       </c>
       <c r="D336" s="7" t="inlineStr"/>
       <c r="E336" s="7" t="inlineStr"/>
-      <c r="F336" s="7" t="inlineStr"/>
+      <c r="F336" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G336" s="7" t="inlineStr"/>
     </row>
     <row r="337">
@@ -6802,7 +7471,9 @@
       </c>
       <c r="D337" s="7" t="inlineStr"/>
       <c r="E337" s="7" t="inlineStr"/>
-      <c r="F337" s="7" t="inlineStr"/>
+      <c r="F337" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G337" s="7" t="inlineStr"/>
     </row>
     <row r="338">
@@ -6821,7 +7492,9 @@
       </c>
       <c r="D338" s="7" t="inlineStr"/>
       <c r="E338" s="7" t="inlineStr"/>
-      <c r="F338" s="7" t="inlineStr"/>
+      <c r="F338" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G338" s="7" t="inlineStr"/>
     </row>
     <row r="339">
@@ -6840,7 +7513,9 @@
       </c>
       <c r="D339" s="7" t="inlineStr"/>
       <c r="E339" s="7" t="inlineStr"/>
-      <c r="F339" s="7" t="inlineStr"/>
+      <c r="F339" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G339" s="7" t="inlineStr"/>
     </row>
     <row r="340">
@@ -6859,7 +7534,9 @@
       </c>
       <c r="D340" s="7" t="inlineStr"/>
       <c r="E340" s="7" t="inlineStr"/>
-      <c r="F340" s="7" t="inlineStr"/>
+      <c r="F340" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G340" s="7" t="inlineStr"/>
     </row>
     <row r="341">
@@ -6878,7 +7555,9 @@
       </c>
       <c r="D341" s="7" t="inlineStr"/>
       <c r="E341" s="7" t="inlineStr"/>
-      <c r="F341" s="7" t="inlineStr"/>
+      <c r="F341" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G341" s="7" t="inlineStr"/>
     </row>
     <row r="342">
@@ -6897,7 +7576,9 @@
       </c>
       <c r="D342" s="7" t="inlineStr"/>
       <c r="E342" s="7" t="inlineStr"/>
-      <c r="F342" s="7" t="inlineStr"/>
+      <c r="F342" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G342" s="7" t="inlineStr"/>
     </row>
     <row r="343">
@@ -6916,7 +7597,9 @@
       </c>
       <c r="D343" s="7" t="inlineStr"/>
       <c r="E343" s="7" t="inlineStr"/>
-      <c r="F343" s="7" t="inlineStr"/>
+      <c r="F343" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G343" s="7" t="inlineStr"/>
     </row>
     <row r="344">
@@ -6935,7 +7618,9 @@
       </c>
       <c r="D344" s="7" t="inlineStr"/>
       <c r="E344" s="7" t="inlineStr"/>
-      <c r="F344" s="7" t="inlineStr"/>
+      <c r="F344" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G344" s="7" t="inlineStr"/>
     </row>
     <row r="345">
@@ -6954,7 +7639,9 @@
       </c>
       <c r="D345" s="7" t="inlineStr"/>
       <c r="E345" s="7" t="inlineStr"/>
-      <c r="F345" s="7" t="inlineStr"/>
+      <c r="F345" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G345" s="7" t="inlineStr"/>
     </row>
     <row r="346">
@@ -6973,7 +7660,9 @@
       </c>
       <c r="D346" s="7" t="inlineStr"/>
       <c r="E346" s="7" t="inlineStr"/>
-      <c r="F346" s="7" t="inlineStr"/>
+      <c r="F346" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G346" s="7" t="inlineStr"/>
     </row>
     <row r="347">
@@ -6992,7 +7681,9 @@
       </c>
       <c r="D347" s="7" t="inlineStr"/>
       <c r="E347" s="7" t="inlineStr"/>
-      <c r="F347" s="7" t="inlineStr"/>
+      <c r="F347" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G347" s="7" t="inlineStr"/>
     </row>
     <row r="348">
@@ -7011,7 +7702,9 @@
       </c>
       <c r="D348" s="7" t="inlineStr"/>
       <c r="E348" s="7" t="inlineStr"/>
-      <c r="F348" s="7" t="inlineStr"/>
+      <c r="F348" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G348" s="7" t="inlineStr"/>
     </row>
     <row r="349">
@@ -7030,7 +7723,9 @@
       </c>
       <c r="D349" s="7" t="inlineStr"/>
       <c r="E349" s="7" t="inlineStr"/>
-      <c r="F349" s="7" t="inlineStr"/>
+      <c r="F349" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G349" s="7" t="inlineStr"/>
     </row>
     <row r="350">
@@ -7049,7 +7744,9 @@
       </c>
       <c r="D350" s="7" t="inlineStr"/>
       <c r="E350" s="7" t="inlineStr"/>
-      <c r="F350" s="7" t="inlineStr"/>
+      <c r="F350" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G350" s="7" t="inlineStr"/>
     </row>
     <row r="351">
@@ -7068,7 +7765,9 @@
       </c>
       <c r="D351" s="7" t="inlineStr"/>
       <c r="E351" s="7" t="inlineStr"/>
-      <c r="F351" s="7" t="inlineStr"/>
+      <c r="F351" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G351" s="7" t="inlineStr"/>
     </row>
     <row r="352">
@@ -7087,7 +7786,9 @@
       </c>
       <c r="D352" s="7" t="inlineStr"/>
       <c r="E352" s="7" t="inlineStr"/>
-      <c r="F352" s="7" t="inlineStr"/>
+      <c r="F352" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G352" s="7" t="inlineStr"/>
     </row>
     <row r="353">
@@ -7106,7 +7807,9 @@
       </c>
       <c r="D353" s="7" t="inlineStr"/>
       <c r="E353" s="7" t="inlineStr"/>
-      <c r="F353" s="7" t="inlineStr"/>
+      <c r="F353" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G353" s="7" t="inlineStr"/>
     </row>
     <row r="354">
@@ -7121,7 +7824,9 @@
       <c r="C354" s="5" t="inlineStr"/>
       <c r="D354" s="7" t="inlineStr"/>
       <c r="E354" s="7" t="inlineStr"/>
-      <c r="F354" s="7" t="inlineStr"/>
+      <c r="F354" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G354" s="7" t="inlineStr"/>
     </row>
     <row r="355">
@@ -7140,7 +7845,9 @@
       </c>
       <c r="D355" s="7" t="inlineStr"/>
       <c r="E355" s="7" t="inlineStr"/>
-      <c r="F355" s="7" t="inlineStr"/>
+      <c r="F355" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="G355" s="7" t="inlineStr"/>
     </row>
     <row r="356">
@@ -7159,7 +7866,9 @@
       </c>
       <c r="D356" s="10" t="inlineStr"/>
       <c r="E356" s="10" t="inlineStr"/>
-      <c r="F356" s="10" t="inlineStr"/>
+      <c r="F356" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G356" s="10" t="inlineStr"/>
     </row>
     <row r="357">
@@ -7178,7 +7887,9 @@
       </c>
       <c r="D357" s="10" t="inlineStr"/>
       <c r="E357" s="10" t="inlineStr"/>
-      <c r="F357" s="10" t="inlineStr"/>
+      <c r="F357" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G357" s="10" t="inlineStr"/>
     </row>
     <row r="358">
@@ -7197,7 +7908,9 @@
       </c>
       <c r="D358" s="10" t="inlineStr"/>
       <c r="E358" s="10" t="inlineStr"/>
-      <c r="F358" s="10" t="inlineStr"/>
+      <c r="F358" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G358" s="10" t="inlineStr"/>
     </row>
     <row r="359">
@@ -7216,7 +7929,9 @@
       </c>
       <c r="D359" s="10" t="inlineStr"/>
       <c r="E359" s="10" t="inlineStr"/>
-      <c r="F359" s="10" t="inlineStr"/>
+      <c r="F359" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G359" s="10" t="inlineStr"/>
     </row>
     <row r="360">
@@ -7235,7 +7950,9 @@
       </c>
       <c r="D360" s="10" t="inlineStr"/>
       <c r="E360" s="10" t="inlineStr"/>
-      <c r="F360" s="10" t="inlineStr"/>
+      <c r="F360" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G360" s="10" t="inlineStr"/>
     </row>
     <row r="361">
@@ -7254,7 +7971,9 @@
       </c>
       <c r="D361" s="10" t="inlineStr"/>
       <c r="E361" s="10" t="inlineStr"/>
-      <c r="F361" s="10" t="inlineStr"/>
+      <c r="F361" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G361" s="10" t="inlineStr"/>
     </row>
     <row r="362">
@@ -7273,7 +7992,9 @@
       </c>
       <c r="D362" s="10" t="inlineStr"/>
       <c r="E362" s="10" t="inlineStr"/>
-      <c r="F362" s="10" t="inlineStr"/>
+      <c r="F362" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G362" s="10" t="inlineStr"/>
     </row>
     <row r="363">
@@ -7292,7 +8013,9 @@
       </c>
       <c r="D363" s="10" t="inlineStr"/>
       <c r="E363" s="10" t="inlineStr"/>
-      <c r="F363" s="10" t="inlineStr"/>
+      <c r="F363" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G363" s="10" t="inlineStr"/>
     </row>
     <row r="364">
@@ -7311,7 +8034,9 @@
       </c>
       <c r="D364" s="10" t="inlineStr"/>
       <c r="E364" s="10" t="inlineStr"/>
-      <c r="F364" s="10" t="inlineStr"/>
+      <c r="F364" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G364" s="10" t="inlineStr"/>
     </row>
     <row r="365">
@@ -7330,7 +8055,9 @@
       </c>
       <c r="D365" s="10" t="inlineStr"/>
       <c r="E365" s="10" t="inlineStr"/>
-      <c r="F365" s="10" t="inlineStr"/>
+      <c r="F365" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G365" s="10" t="inlineStr"/>
     </row>
     <row r="366">
@@ -7349,7 +8076,9 @@
       </c>
       <c r="D366" s="10" t="inlineStr"/>
       <c r="E366" s="10" t="inlineStr"/>
-      <c r="F366" s="10" t="inlineStr"/>
+      <c r="F366" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G366" s="10" t="inlineStr"/>
     </row>
     <row r="367">
@@ -7368,7 +8097,9 @@
       </c>
       <c r="D367" s="10" t="inlineStr"/>
       <c r="E367" s="10" t="inlineStr"/>
-      <c r="F367" s="10" t="inlineStr"/>
+      <c r="F367" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G367" s="10" t="inlineStr"/>
     </row>
     <row r="368">
@@ -7387,7 +8118,9 @@
       </c>
       <c r="D368" s="10" t="inlineStr"/>
       <c r="E368" s="10" t="inlineStr"/>
-      <c r="F368" s="10" t="inlineStr"/>
+      <c r="F368" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G368" s="10" t="inlineStr"/>
     </row>
     <row r="369">
@@ -7406,7 +8139,9 @@
       </c>
       <c r="D369" s="10" t="inlineStr"/>
       <c r="E369" s="10" t="inlineStr"/>
-      <c r="F369" s="10" t="inlineStr"/>
+      <c r="F369" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G369" s="10" t="inlineStr"/>
     </row>
     <row r="370">
@@ -7425,7 +8160,9 @@
       </c>
       <c r="D370" s="10" t="inlineStr"/>
       <c r="E370" s="10" t="inlineStr"/>
-      <c r="F370" s="10" t="inlineStr"/>
+      <c r="F370" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G370" s="10" t="inlineStr"/>
     </row>
     <row r="371">
@@ -7444,7 +8181,9 @@
       </c>
       <c r="D371" s="10" t="inlineStr"/>
       <c r="E371" s="10" t="inlineStr"/>
-      <c r="F371" s="10" t="inlineStr"/>
+      <c r="F371" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G371" s="10" t="inlineStr"/>
     </row>
     <row r="372">
@@ -7463,7 +8202,9 @@
       </c>
       <c r="D372" s="10" t="inlineStr"/>
       <c r="E372" s="10" t="inlineStr"/>
-      <c r="F372" s="10" t="inlineStr"/>
+      <c r="F372" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G372" s="10" t="inlineStr"/>
     </row>
     <row r="373">
@@ -7482,7 +8223,9 @@
       </c>
       <c r="D373" s="10" t="inlineStr"/>
       <c r="E373" s="10" t="inlineStr"/>
-      <c r="F373" s="10" t="inlineStr"/>
+      <c r="F373" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G373" s="10" t="inlineStr"/>
     </row>
     <row r="374">
@@ -7501,7 +8244,9 @@
       </c>
       <c r="D374" s="10" t="inlineStr"/>
       <c r="E374" s="10" t="inlineStr"/>
-      <c r="F374" s="10" t="inlineStr"/>
+      <c r="F374" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G374" s="10" t="inlineStr"/>
     </row>
     <row r="375">
@@ -7520,7 +8265,9 @@
       </c>
       <c r="D375" s="10" t="inlineStr"/>
       <c r="E375" s="10" t="inlineStr"/>
-      <c r="F375" s="10" t="inlineStr"/>
+      <c r="F375" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G375" s="10" t="inlineStr"/>
     </row>
     <row r="376">
@@ -7539,7 +8286,9 @@
       </c>
       <c r="D376" s="10" t="inlineStr"/>
       <c r="E376" s="10" t="inlineStr"/>
-      <c r="F376" s="10" t="inlineStr"/>
+      <c r="F376" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G376" s="10" t="inlineStr"/>
     </row>
     <row r="377">
@@ -7558,7 +8307,9 @@
       </c>
       <c r="D377" s="10" t="inlineStr"/>
       <c r="E377" s="10" t="inlineStr"/>
-      <c r="F377" s="10" t="inlineStr"/>
+      <c r="F377" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G377" s="10" t="inlineStr"/>
     </row>
     <row r="378">
@@ -7577,7 +8328,9 @@
       </c>
       <c r="D378" s="10" t="inlineStr"/>
       <c r="E378" s="10" t="inlineStr"/>
-      <c r="F378" s="10" t="inlineStr"/>
+      <c r="F378" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G378" s="10" t="inlineStr"/>
     </row>
     <row r="379">
@@ -7596,7 +8349,9 @@
       </c>
       <c r="D379" s="10" t="inlineStr"/>
       <c r="E379" s="10" t="inlineStr"/>
-      <c r="F379" s="10" t="inlineStr"/>
+      <c r="F379" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G379" s="10" t="inlineStr"/>
     </row>
     <row r="380">
@@ -7615,7 +8370,9 @@
       </c>
       <c r="D380" s="10" t="inlineStr"/>
       <c r="E380" s="10" t="inlineStr"/>
-      <c r="F380" s="10" t="inlineStr"/>
+      <c r="F380" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G380" s="10" t="inlineStr"/>
     </row>
     <row r="381">
@@ -7634,7 +8391,9 @@
       </c>
       <c r="D381" s="10" t="inlineStr"/>
       <c r="E381" s="10" t="inlineStr"/>
-      <c r="F381" s="10" t="inlineStr"/>
+      <c r="F381" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G381" s="10" t="inlineStr"/>
     </row>
     <row r="382">
@@ -7653,7 +8412,9 @@
       </c>
       <c r="D382" s="10" t="inlineStr"/>
       <c r="E382" s="10" t="inlineStr"/>
-      <c r="F382" s="10" t="inlineStr"/>
+      <c r="F382" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G382" s="10" t="inlineStr"/>
     </row>
     <row r="383">
@@ -7672,7 +8433,9 @@
       </c>
       <c r="D383" s="10" t="inlineStr"/>
       <c r="E383" s="10" t="inlineStr"/>
-      <c r="F383" s="10" t="inlineStr"/>
+      <c r="F383" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G383" s="10" t="inlineStr"/>
     </row>
     <row r="384">
@@ -7691,7 +8454,9 @@
       </c>
       <c r="D384" s="10" t="inlineStr"/>
       <c r="E384" s="10" t="inlineStr"/>
-      <c r="F384" s="10" t="inlineStr"/>
+      <c r="F384" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G384" s="10" t="inlineStr"/>
     </row>
     <row r="385">
@@ -7710,7 +8475,9 @@
       </c>
       <c r="D385" s="10" t="inlineStr"/>
       <c r="E385" s="10" t="inlineStr"/>
-      <c r="F385" s="10" t="inlineStr"/>
+      <c r="F385" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G385" s="10" t="inlineStr"/>
     </row>
     <row r="386">
@@ -7725,7 +8492,9 @@
       <c r="C386" s="8" t="inlineStr"/>
       <c r="D386" s="10" t="inlineStr"/>
       <c r="E386" s="10" t="inlineStr"/>
-      <c r="F386" s="10" t="inlineStr"/>
+      <c r="F386" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G386" s="10" t="inlineStr"/>
     </row>
     <row r="387">
@@ -7740,7 +8509,9 @@
       <c r="C387" s="8" t="inlineStr"/>
       <c r="D387" s="10" t="inlineStr"/>
       <c r="E387" s="10" t="inlineStr"/>
-      <c r="F387" s="10" t="inlineStr"/>
+      <c r="F387" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G387" s="10" t="inlineStr"/>
     </row>
     <row r="388">
@@ -7755,7 +8526,9 @@
       <c r="C388" s="8" t="inlineStr"/>
       <c r="D388" s="10" t="inlineStr"/>
       <c r="E388" s="10" t="inlineStr"/>
-      <c r="F388" s="10" t="inlineStr"/>
+      <c r="F388" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G388" s="10" t="inlineStr"/>
     </row>
     <row r="389">
@@ -7770,7 +8543,9 @@
       <c r="C389" s="8" t="inlineStr"/>
       <c r="D389" s="10" t="inlineStr"/>
       <c r="E389" s="10" t="inlineStr"/>
-      <c r="F389" s="10" t="inlineStr"/>
+      <c r="F389" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G389" s="10" t="inlineStr"/>
     </row>
     <row r="390">
@@ -7785,7 +8560,9 @@
       <c r="C390" s="8" t="inlineStr"/>
       <c r="D390" s="10" t="inlineStr"/>
       <c r="E390" s="10" t="inlineStr"/>
-      <c r="F390" s="10" t="inlineStr"/>
+      <c r="F390" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G390" s="10" t="inlineStr"/>
     </row>
     <row r="391">
@@ -7800,7 +8577,9 @@
       <c r="C391" s="8" t="inlineStr"/>
       <c r="D391" s="10" t="inlineStr"/>
       <c r="E391" s="10" t="inlineStr"/>
-      <c r="F391" s="10" t="inlineStr"/>
+      <c r="F391" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G391" s="10" t="inlineStr"/>
     </row>
     <row r="392">
@@ -7815,7 +8594,9 @@
       <c r="C392" s="8" t="inlineStr"/>
       <c r="D392" s="10" t="inlineStr"/>
       <c r="E392" s="10" t="inlineStr"/>
-      <c r="F392" s="10" t="inlineStr"/>
+      <c r="F392" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G392" s="10" t="inlineStr"/>
     </row>
     <row r="393">
@@ -7830,7 +8611,9 @@
       <c r="C393" s="8" t="inlineStr"/>
       <c r="D393" s="10" t="inlineStr"/>
       <c r="E393" s="10" t="inlineStr"/>
-      <c r="F393" s="10" t="inlineStr"/>
+      <c r="F393" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G393" s="10" t="inlineStr"/>
     </row>
     <row r="394">
@@ -7845,7 +8628,9 @@
       <c r="C394" s="8" t="inlineStr"/>
       <c r="D394" s="10" t="inlineStr"/>
       <c r="E394" s="10" t="inlineStr"/>
-      <c r="F394" s="10" t="inlineStr"/>
+      <c r="F394" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G394" s="10" t="inlineStr"/>
     </row>
     <row r="395">
@@ -7860,7 +8645,9 @@
       <c r="C395" s="8" t="inlineStr"/>
       <c r="D395" s="10" t="inlineStr"/>
       <c r="E395" s="10" t="inlineStr"/>
-      <c r="F395" s="10" t="inlineStr"/>
+      <c r="F395" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G395" s="10" t="inlineStr"/>
     </row>
     <row r="396">
@@ -7875,7 +8662,9 @@
       <c r="C396" s="8" t="inlineStr"/>
       <c r="D396" s="10" t="inlineStr"/>
       <c r="E396" s="10" t="inlineStr"/>
-      <c r="F396" s="10" t="inlineStr"/>
+      <c r="F396" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G396" s="10" t="inlineStr"/>
     </row>
     <row r="397">
@@ -7890,7 +8679,9 @@
       <c r="C397" s="8" t="inlineStr"/>
       <c r="D397" s="10" t="inlineStr"/>
       <c r="E397" s="10" t="inlineStr"/>
-      <c r="F397" s="10" t="inlineStr"/>
+      <c r="F397" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G397" s="10" t="inlineStr"/>
     </row>
     <row r="398">
@@ -7905,7 +8696,9 @@
       <c r="C398" s="8" t="inlineStr"/>
       <c r="D398" s="10" t="inlineStr"/>
       <c r="E398" s="10" t="inlineStr"/>
-      <c r="F398" s="10" t="inlineStr"/>
+      <c r="F398" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G398" s="10" t="inlineStr"/>
     </row>
     <row r="399">
@@ -7920,7 +8713,9 @@
       <c r="C399" s="8" t="inlineStr"/>
       <c r="D399" s="10" t="inlineStr"/>
       <c r="E399" s="10" t="inlineStr"/>
-      <c r="F399" s="10" t="inlineStr"/>
+      <c r="F399" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G399" s="10" t="inlineStr"/>
     </row>
     <row r="400">
@@ -7935,7 +8730,9 @@
       <c r="C400" s="8" t="inlineStr"/>
       <c r="D400" s="10" t="inlineStr"/>
       <c r="E400" s="10" t="inlineStr"/>
-      <c r="F400" s="10" t="inlineStr"/>
+      <c r="F400" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G400" s="10" t="inlineStr"/>
     </row>
     <row r="401">
@@ -7950,7 +8747,9 @@
       <c r="C401" s="8" t="inlineStr"/>
       <c r="D401" s="10" t="inlineStr"/>
       <c r="E401" s="10" t="inlineStr"/>
-      <c r="F401" s="10" t="inlineStr"/>
+      <c r="F401" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G401" s="10" t="inlineStr"/>
     </row>
     <row r="402">
@@ -7965,7 +8764,9 @@
       <c r="C402" s="8" t="inlineStr"/>
       <c r="D402" s="10" t="inlineStr"/>
       <c r="E402" s="10" t="inlineStr"/>
-      <c r="F402" s="10" t="inlineStr"/>
+      <c r="F402" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G402" s="10" t="inlineStr"/>
     </row>
     <row r="403">
@@ -7980,7 +8781,9 @@
       <c r="C403" s="8" t="inlineStr"/>
       <c r="D403" s="10" t="inlineStr"/>
       <c r="E403" s="10" t="inlineStr"/>
-      <c r="F403" s="10" t="inlineStr"/>
+      <c r="F403" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G403" s="10" t="inlineStr"/>
     </row>
     <row r="404">
@@ -7995,7 +8798,9 @@
       <c r="C404" s="8" t="inlineStr"/>
       <c r="D404" s="10" t="inlineStr"/>
       <c r="E404" s="10" t="inlineStr"/>
-      <c r="F404" s="10" t="inlineStr"/>
+      <c r="F404" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G404" s="10" t="inlineStr"/>
     </row>
     <row r="405">
@@ -8010,7 +8815,9 @@
       <c r="C405" s="8" t="inlineStr"/>
       <c r="D405" s="10" t="inlineStr"/>
       <c r="E405" s="10" t="inlineStr"/>
-      <c r="F405" s="10" t="inlineStr"/>
+      <c r="F405" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G405" s="10" t="inlineStr"/>
     </row>
     <row r="406">
@@ -8025,7 +8832,9 @@
       <c r="C406" s="8" t="inlineStr"/>
       <c r="D406" s="10" t="inlineStr"/>
       <c r="E406" s="10" t="inlineStr"/>
-      <c r="F406" s="10" t="inlineStr"/>
+      <c r="F406" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G406" s="10" t="inlineStr"/>
     </row>
     <row r="407">
@@ -8040,7 +8849,9 @@
       <c r="C407" s="8" t="inlineStr"/>
       <c r="D407" s="10" t="inlineStr"/>
       <c r="E407" s="10" t="inlineStr"/>
-      <c r="F407" s="10" t="inlineStr"/>
+      <c r="F407" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G407" s="10" t="inlineStr"/>
     </row>
     <row r="408">
@@ -8055,7 +8866,9 @@
       <c r="C408" s="8" t="inlineStr"/>
       <c r="D408" s="10" t="inlineStr"/>
       <c r="E408" s="10" t="inlineStr"/>
-      <c r="F408" s="10" t="inlineStr"/>
+      <c r="F408" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G408" s="10" t="inlineStr"/>
     </row>
     <row r="409">
@@ -8074,7 +8887,9 @@
       </c>
       <c r="D409" s="10" t="inlineStr"/>
       <c r="E409" s="10" t="inlineStr"/>
-      <c r="F409" s="10" t="inlineStr"/>
+      <c r="F409" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G409" s="10" t="inlineStr"/>
     </row>
     <row r="410">
@@ -8093,7 +8908,9 @@
       </c>
       <c r="D410" s="10" t="inlineStr"/>
       <c r="E410" s="10" t="inlineStr"/>
-      <c r="F410" s="10" t="inlineStr"/>
+      <c r="F410" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G410" s="10" t="inlineStr"/>
     </row>
     <row r="411">
@@ -8112,7 +8929,9 @@
       </c>
       <c r="D411" s="10" t="inlineStr"/>
       <c r="E411" s="10" t="inlineStr"/>
-      <c r="F411" s="10" t="inlineStr"/>
+      <c r="F411" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G411" s="10" t="inlineStr"/>
     </row>
     <row r="412">
@@ -8131,7 +8950,9 @@
       </c>
       <c r="D412" s="10" t="inlineStr"/>
       <c r="E412" s="10" t="inlineStr"/>
-      <c r="F412" s="10" t="inlineStr"/>
+      <c r="F412" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G412" s="10" t="inlineStr"/>
     </row>
     <row r="413">
@@ -8150,7 +8971,9 @@
       </c>
       <c r="D413" s="10" t="inlineStr"/>
       <c r="E413" s="10" t="inlineStr"/>
-      <c r="F413" s="10" t="inlineStr"/>
+      <c r="F413" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G413" s="10" t="inlineStr"/>
     </row>
     <row r="414">
@@ -8169,7 +8992,9 @@
       </c>
       <c r="D414" s="10" t="inlineStr"/>
       <c r="E414" s="10" t="inlineStr"/>
-      <c r="F414" s="10" t="inlineStr"/>
+      <c r="F414" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G414" s="10" t="inlineStr"/>
     </row>
     <row r="415">
@@ -8188,7 +9013,9 @@
       </c>
       <c r="D415" s="10" t="inlineStr"/>
       <c r="E415" s="10" t="inlineStr"/>
-      <c r="F415" s="10" t="inlineStr"/>
+      <c r="F415" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G415" s="10" t="inlineStr"/>
     </row>
     <row r="416">
@@ -8207,7 +9034,9 @@
       </c>
       <c r="D416" s="10" t="inlineStr"/>
       <c r="E416" s="10" t="inlineStr"/>
-      <c r="F416" s="10" t="inlineStr"/>
+      <c r="F416" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G416" s="10" t="inlineStr"/>
     </row>
     <row r="417">
@@ -8226,7 +9055,9 @@
       </c>
       <c r="D417" s="10" t="inlineStr"/>
       <c r="E417" s="10" t="inlineStr"/>
-      <c r="F417" s="10" t="inlineStr"/>
+      <c r="F417" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G417" s="10" t="inlineStr"/>
     </row>
     <row r="418">
@@ -8245,7 +9076,9 @@
       </c>
       <c r="D418" s="10" t="inlineStr"/>
       <c r="E418" s="10" t="inlineStr"/>
-      <c r="F418" s="10" t="inlineStr"/>
+      <c r="F418" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G418" s="10" t="inlineStr"/>
     </row>
     <row r="419">
@@ -8264,7 +9097,9 @@
       </c>
       <c r="D419" s="10" t="inlineStr"/>
       <c r="E419" s="10" t="inlineStr"/>
-      <c r="F419" s="10" t="inlineStr"/>
+      <c r="F419" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G419" s="10" t="inlineStr"/>
     </row>
     <row r="420">
@@ -8283,7 +9118,9 @@
       </c>
       <c r="D420" s="10" t="inlineStr"/>
       <c r="E420" s="10" t="inlineStr"/>
-      <c r="F420" s="10" t="inlineStr"/>
+      <c r="F420" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G420" s="10" t="inlineStr"/>
     </row>
     <row r="421">
@@ -8302,7 +9139,9 @@
       </c>
       <c r="D421" s="10" t="inlineStr"/>
       <c r="E421" s="10" t="inlineStr"/>
-      <c r="F421" s="10" t="inlineStr"/>
+      <c r="F421" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G421" s="10" t="inlineStr"/>
     </row>
     <row r="422">
@@ -8321,180 +9160,28 @@
       </c>
       <c r="D422" s="10" t="inlineStr"/>
       <c r="E422" s="10" t="inlineStr"/>
-      <c r="F422" s="10" t="inlineStr"/>
+      <c r="F422" s="10" t="b">
+        <v>0</v>
+      </c>
       <c r="G422" s="10" t="inlineStr"/>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
   <conditionalFormatting sqref="A2:G422">
     <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="0">
       <formula>OR($D2="",AND($E2&lt;&gt;"",$E2=$D2),AND($E2&lt;&gt;"",OR($D2="No Distortion",$D2="No Distortion (calibrated pessimism)")))</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation sqref="D2:D422" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>_lists!$A$1:$A$12</formula1>
+    <dataValidation sqref="D2:D422" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="Pick from the list" error="Choose one of the labels in the dropdown." promptTitle="Primary" prompt="Required. One label." type="list">
+      <formula1>"All-or-nothing thinking,Emotional Reasoning,Fortune-telling,Labeling,Magnification,Mental filter,Mind Reading,No Distortion,Overgeneralization,Personalization,Should statements,No Distortion (calibrated pessimism)"</formula1>
     </dataValidation>
-    <dataValidation sqref="E2:E422" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>_lists!$B$1:$B$10</formula1>
+    <dataValidation sqref="E2:E422" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Choose one of the ten distortions, or leave blank." type="list">
+      <formula1>"All-or-nothing thinking,Emotional Reasoning,Fortune-telling,Labeling,Magnification,Mental filter,Mind Reading,Overgeneralization,Personalization,Should statements"</formula1>
     </dataValidation>
     <dataValidation sqref="F2:F422" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>_lists!$C$1:$C$1</formula1>
+      <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>All-or-nothing thinking</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>All-or-nothing thinking</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Emotional Reasoning</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Emotional Reasoning</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Fortune-telling</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Fortune-telling</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Labeling</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Labeling</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Magnification</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Magnification</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Mental filter</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Mental filter</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Mind Reading</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Mind Reading</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>No Distortion</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Overgeneralization</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Overgeneralization</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Personalization</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Personalization</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Should statements</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Should statements</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>No Distortion (calibrated pessimism)</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>